<commit_message>
Add Skyeview Mesa concrete (10/1/2026 PPS) and SL Lark Hill concrete (7/1/2025 TM schedule)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D6wjrb1spFgY1HgqZrWwPC
</commit_message>
<xml_diff>
--- a/CenturyCommunitiesContracts1.xlsx
+++ b/CenturyCommunitiesContracts1.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F188"/>
+  <dimension ref="A1:F196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5697,6 +5697,230 @@
         <v>3210</v>
       </c>
     </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Skyeview - Mesa - Concrete</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C189" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>1635</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="n">
+        <v>8567</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Skyeview - Mesa - Concrete</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C190" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>1635</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="n">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Skyeview - Mesa - Concrete</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C191" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>1742</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="n">
+        <v>8926</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Skyeview - Mesa - Concrete</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C192" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>1742</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="n">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Skyeview - Mesa - Concrete</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C193" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>1816</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="n">
+        <v>9330</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Skyeview - Mesa - Concrete</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C194" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>1816</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="n">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Skyeview - Mesa - Concrete</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C195" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>1635</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>BED0030 - Bedroom 3/Bath</t>
+        </is>
+      </c>
+      <c r="F195" s="2" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Skyeview - Mesa - Concrete</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C196" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>1816</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>BED0040 - Bedroom 4/Bath</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="n">
+        <v>300</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add SupplyPro-paid prices for Ishani Ridge, Esplanade Duplex concrete, Portofino 40s/50s/60s pavers, MF 40s
New contract dates carry the Note "Price reduced from contract approved by Tony"; original contract prices kept as historical.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D6wjrb1spFgY1HgqZrWwPC
</commit_message>
<xml_diff>
--- a/CenturyCommunitiesContracts1.xlsx
+++ b/CenturyCommunitiesContracts1.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F196"/>
+  <dimension ref="A1:G197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -427,6 +427,7 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,6 +461,11 @@
           <t>Amount</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -488,6 +494,7 @@
       <c r="F2" s="2" t="n">
         <v>6450</v>
       </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -516,6 +523,7 @@
       <c r="F3" s="2" t="n">
         <v>6788</v>
       </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -544,6 +552,7 @@
       <c r="F4" s="2" t="n">
         <v>6788</v>
       </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -572,6 +581,7 @@
       <c r="F5" s="2" t="n">
         <v>6791</v>
       </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -600,6 +610,7 @@
       <c r="F6" s="2" t="n">
         <v>6704</v>
       </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -628,6 +639,7 @@
       <c r="F7" s="2" t="n">
         <v>555</v>
       </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -656,6 +668,7 @@
       <c r="F8" s="2" t="n">
         <v>6596</v>
       </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -684,6 +697,7 @@
       <c r="F9" s="2" t="n">
         <v>580</v>
       </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -712,6 +726,7 @@
       <c r="F10" s="2" t="n">
         <v>7112</v>
       </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -740,6 +755,7 @@
       <c r="F11" s="2" t="n">
         <v>580</v>
       </c>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -768,6 +784,7 @@
       <c r="F12" s="2" t="n">
         <v>6966</v>
       </c>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -796,6 +813,7 @@
       <c r="F13" s="2" t="n">
         <v>581</v>
       </c>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -824,6 +842,7 @@
       <c r="F14" s="2" t="n">
         <v>581</v>
       </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -852,6 +871,7 @@
       <c r="F15" s="2" t="n">
         <v>581</v>
       </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -880,6 +900,7 @@
       <c r="F16" s="2" t="n">
         <v>581</v>
       </c>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -908,6 +929,7 @@
       <c r="F17" s="2" t="n">
         <v>581</v>
       </c>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -936,6 +958,7 @@
       <c r="F18" s="2" t="n">
         <v>7162</v>
       </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -964,6 +987,7 @@
       <c r="F19" s="2" t="n">
         <v>579</v>
       </c>
+      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -992,6 +1016,7 @@
       <c r="F20" s="2" t="n">
         <v>579</v>
       </c>
+      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1020,6 +1045,7 @@
       <c r="F21" s="2" t="n">
         <v>579</v>
       </c>
+      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1048,6 +1074,7 @@
       <c r="F22" s="2" t="n">
         <v>579</v>
       </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1076,6 +1103,7 @@
       <c r="F23" s="2" t="n">
         <v>579</v>
       </c>
+      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1104,6 +1132,7 @@
       <c r="F24" s="2" t="n">
         <v>7096</v>
       </c>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1132,6 +1161,7 @@
       <c r="F25" s="2" t="n">
         <v>549</v>
       </c>
+      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1160,6 +1190,7 @@
       <c r="F26" s="2" t="n">
         <v>549</v>
       </c>
+      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1188,6 +1219,7 @@
       <c r="F27" s="2" t="n">
         <v>549</v>
       </c>
+      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1216,6 +1248,7 @@
       <c r="F28" s="2" t="n">
         <v>549</v>
       </c>
+      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1244,6 +1277,7 @@
       <c r="F29" s="2" t="n">
         <v>7802</v>
       </c>
+      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1272,6 +1306,7 @@
       <c r="F30" s="2" t="n">
         <v>588</v>
       </c>
+      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1300,6 +1335,7 @@
       <c r="F31" s="2" t="n">
         <v>588</v>
       </c>
+      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1328,6 +1364,7 @@
       <c r="F32" s="2" t="n">
         <v>588</v>
       </c>
+      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1356,6 +1393,7 @@
       <c r="F33" s="2" t="n">
         <v>549</v>
       </c>
+      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1384,6 +1422,7 @@
       <c r="F34" s="2" t="n">
         <v>588</v>
       </c>
+      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1412,6 +1451,7 @@
       <c r="F35" s="2" t="n">
         <v>7270</v>
       </c>
+      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1440,6 +1480,7 @@
       <c r="F36" s="2" t="n">
         <v>702</v>
       </c>
+      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1468,6 +1509,7 @@
       <c r="F37" s="2" t="n">
         <v>702</v>
       </c>
+      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1496,6 +1538,7 @@
       <c r="F38" s="2" t="n">
         <v>702</v>
       </c>
+      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1524,6 +1567,7 @@
       <c r="F39" s="2" t="n">
         <v>702</v>
       </c>
+      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1552,6 +1596,7 @@
       <c r="F40" s="2" t="n">
         <v>702</v>
       </c>
+      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1580,6 +1625,7 @@
       <c r="F41" s="2" t="n">
         <v>7450</v>
       </c>
+      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1608,6 +1654,7 @@
       <c r="F42" s="2" t="n">
         <v>513</v>
       </c>
+      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1636,6 +1683,7 @@
       <c r="F43" s="2" t="n">
         <v>513</v>
       </c>
+      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1664,6 +1712,7 @@
       <c r="F44" s="2" t="n">
         <v>513</v>
       </c>
+      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1692,6 +1741,7 @@
       <c r="F45" s="2" t="n">
         <v>513</v>
       </c>
+      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1720,6 +1770,7 @@
       <c r="F46" s="2" t="n">
         <v>513</v>
       </c>
+      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1748,6 +1799,7 @@
       <c r="F47" s="2" t="n">
         <v>7713</v>
       </c>
+      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1776,6 +1828,7 @@
       <c r="F48" s="2" t="n">
         <v>504</v>
       </c>
+      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1804,6 +1857,7 @@
       <c r="F49" s="2" t="n">
         <v>504</v>
       </c>
+      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1832,6 +1886,7 @@
       <c r="F50" s="2" t="n">
         <v>504</v>
       </c>
+      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1860,6 +1915,7 @@
       <c r="F51" s="2" t="n">
         <v>504</v>
       </c>
+      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1888,6 +1944,7 @@
       <c r="F52" s="2" t="n">
         <v>504</v>
       </c>
+      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1916,6 +1973,7 @@
       <c r="F53" s="2" t="n">
         <v>6295</v>
       </c>
+      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1944,6 +2002,7 @@
       <c r="F54" s="2" t="n">
         <v>6665</v>
       </c>
+      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1972,6 +2031,7 @@
       <c r="F55" s="2" t="n">
         <v>7324</v>
       </c>
+      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2000,6 +2060,7 @@
       <c r="F56" s="2" t="n">
         <v>6434</v>
       </c>
+      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2028,6 +2089,7 @@
       <c r="F57" s="2" t="n">
         <v>541</v>
       </c>
+      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2056,6 +2118,7 @@
       <c r="F58" s="2" t="n">
         <v>6755</v>
       </c>
+      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2084,6 +2147,7 @@
       <c r="F59" s="2" t="n">
         <v>541</v>
       </c>
+      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2112,6 +2176,7 @@
       <c r="F60" s="2" t="n">
         <v>6989</v>
       </c>
+      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2140,6 +2205,7 @@
       <c r="F61" s="2" t="n">
         <v>525</v>
       </c>
+      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2168,6 +2234,7 @@
       <c r="F62" s="2" t="n">
         <v>6630</v>
       </c>
+      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2196,6 +2263,7 @@
       <c r="F63" s="2" t="n">
         <v>350</v>
       </c>
+      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2224,6 +2292,7 @@
       <c r="F64" s="2" t="n">
         <v>7194</v>
       </c>
+      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2252,6 +2321,7 @@
       <c r="F65" s="2" t="n">
         <v>350</v>
       </c>
+      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2280,6 +2350,7 @@
       <c r="F66" s="2" t="n">
         <v>7575</v>
       </c>
+      <c r="G66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2308,6 +2379,7 @@
       <c r="F67" s="2" t="n">
         <v>350</v>
       </c>
+      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2336,6 +2408,7 @@
       <c r="F68" s="2" t="n">
         <v>3012</v>
       </c>
+      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2364,6 +2437,7 @@
       <c r="F69" s="2" t="n">
         <v>4216</v>
       </c>
+      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2392,6 +2466,7 @@
       <c r="F70" s="2" t="n">
         <v>1804</v>
       </c>
+      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2420,6 +2495,7 @@
       <c r="F71" s="2" t="n">
         <v>720</v>
       </c>
+      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2448,6 +2524,7 @@
       <c r="F72" s="2" t="n">
         <v>960</v>
       </c>
+      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2476,6 +2553,7 @@
       <c r="F73" s="2" t="n">
         <v>480</v>
       </c>
+      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2504,6 +2582,7 @@
       <c r="F74" s="2" t="n">
         <v>660</v>
       </c>
+      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2532,6 +2611,7 @@
       <c r="F75" s="2" t="n">
         <v>960</v>
       </c>
+      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2560,6 +2640,7 @@
       <c r="F76" s="2" t="n">
         <v>480</v>
       </c>
+      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2588,6 +2669,7 @@
       <c r="F77" s="2" t="n">
         <v>2259</v>
       </c>
+      <c r="G77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2616,6 +2698,7 @@
       <c r="F78" s="2" t="n">
         <v>3162</v>
       </c>
+      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2644,6 +2727,7 @@
       <c r="F79" s="2" t="n">
         <v>1353</v>
       </c>
+      <c r="G79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2672,6 +2756,7 @@
       <c r="F80" s="2" t="n">
         <v>540</v>
       </c>
+      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2700,6 +2785,7 @@
       <c r="F81" s="2" t="n">
         <v>720</v>
       </c>
+      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2728,6 +2814,7 @@
       <c r="F82" s="2" t="n">
         <v>360</v>
       </c>
+      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2756,6 +2843,7 @@
       <c r="F83" s="2" t="n">
         <v>495</v>
       </c>
+      <c r="G83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2784,6 +2872,7 @@
       <c r="F84" s="2" t="n">
         <v>720</v>
       </c>
+      <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2812,6 +2901,7 @@
       <c r="F85" s="2" t="n">
         <v>360</v>
       </c>
+      <c r="G85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2840,6 +2930,7 @@
       <c r="F86" s="2" t="n">
         <v>5714</v>
       </c>
+      <c r="G86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2868,6 +2959,7 @@
       <c r="F87" s="2" t="n">
         <v>6012</v>
       </c>
+      <c r="G87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2896,6 +2988,7 @@
       <c r="F88" s="2" t="n">
         <v>6012</v>
       </c>
+      <c r="G88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2924,6 +3017,7 @@
       <c r="F89" s="2" t="n">
         <v>6016</v>
       </c>
+      <c r="G89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2952,6 +3046,7 @@
       <c r="F90" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2980,6 +3075,7 @@
       <c r="F91" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="G91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3008,6 +3104,7 @@
       <c r="F92" s="2" t="n">
         <v>375</v>
       </c>
+      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3036,6 +3133,7 @@
       <c r="F93" s="2" t="n">
         <v>225</v>
       </c>
+      <c r="G93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3064,6 +3162,7 @@
       <c r="F94" s="2" t="n">
         <v>225</v>
       </c>
+      <c r="G94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3092,6 +3191,7 @@
       <c r="F95" s="2" t="n">
         <v>420</v>
       </c>
+      <c r="G95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3120,6 +3220,7 @@
       <c r="F96" s="2" t="n">
         <v>450</v>
       </c>
+      <c r="G96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3148,6 +3249,7 @@
       <c r="F97" s="2" t="n">
         <v>125</v>
       </c>
+      <c r="G97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3176,6 +3278,7 @@
       <c r="F98" s="2" t="n">
         <v>555</v>
       </c>
+      <c r="G98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3204,6 +3307,7 @@
       <c r="F99" s="2" t="n">
         <v>69</v>
       </c>
+      <c r="G99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3232,6 +3336,7 @@
       <c r="F100" s="2" t="n">
         <v>90</v>
       </c>
+      <c r="G100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3260,6 +3365,7 @@
       <c r="F101" s="2" t="n">
         <v>81</v>
       </c>
+      <c r="G101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3288,6 +3394,7 @@
       <c r="F102" s="2" t="n">
         <v>13.5</v>
       </c>
+      <c r="G102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3316,6 +3423,7 @@
       <c r="F103" s="2" t="n">
         <v>29.5</v>
       </c>
+      <c r="G103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3344,6 +3452,7 @@
       <c r="F104" s="2" t="n">
         <v>28.5</v>
       </c>
+      <c r="G104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3372,6 +3481,7 @@
       <c r="F105" s="2" t="n">
         <v>105</v>
       </c>
+      <c r="G105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3400,6 +3510,7 @@
       <c r="F106" s="2" t="n">
         <v>240</v>
       </c>
+      <c r="G106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3428,6 +3539,7 @@
       <c r="F107" s="2" t="n">
         <v>850</v>
       </c>
+      <c r="G107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3456,6 +3568,7 @@
       <c r="F108" s="2" t="n">
         <v>2300</v>
       </c>
+      <c r="G108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3484,6 +3597,7 @@
       <c r="F109" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="G109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3512,6 +3626,7 @@
       <c r="F110" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="G110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3540,6 +3655,7 @@
       <c r="F111" s="2" t="n">
         <v>375</v>
       </c>
+      <c r="G111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3568,6 +3684,7 @@
       <c r="F112" s="2" t="n">
         <v>225</v>
       </c>
+      <c r="G112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3596,6 +3713,7 @@
       <c r="F113" s="2" t="n">
         <v>225</v>
       </c>
+      <c r="G113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3624,6 +3742,7 @@
       <c r="F114" s="2" t="n">
         <v>420</v>
       </c>
+      <c r="G114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3652,6 +3771,7 @@
       <c r="F115" s="2" t="n">
         <v>450</v>
       </c>
+      <c r="G115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3680,6 +3800,7 @@
       <c r="F116" s="2" t="n">
         <v>125</v>
       </c>
+      <c r="G116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3708,6 +3829,7 @@
       <c r="F117" s="2" t="n">
         <v>555</v>
       </c>
+      <c r="G117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3736,6 +3858,7 @@
       <c r="F118" s="2" t="n">
         <v>69</v>
       </c>
+      <c r="G118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3764,6 +3887,7 @@
       <c r="F119" s="2" t="n">
         <v>90</v>
       </c>
+      <c r="G119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3792,6 +3916,7 @@
       <c r="F120" s="2" t="n">
         <v>81</v>
       </c>
+      <c r="G120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3820,6 +3945,7 @@
       <c r="F121" s="2" t="n">
         <v>13.5</v>
       </c>
+      <c r="G121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3848,6 +3974,7 @@
       <c r="F122" s="2" t="n">
         <v>29.5</v>
       </c>
+      <c r="G122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3876,6 +4003,7 @@
       <c r="F123" s="2" t="n">
         <v>28.5</v>
       </c>
+      <c r="G123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3904,6 +4032,7 @@
       <c r="F124" s="2" t="n">
         <v>105</v>
       </c>
+      <c r="G124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3932,6 +4061,7 @@
       <c r="F125" s="2" t="n">
         <v>240</v>
       </c>
+      <c r="G125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3960,6 +4090,7 @@
       <c r="F126" s="2" t="n">
         <v>850</v>
       </c>
+      <c r="G126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3988,6 +4119,7 @@
       <c r="F127" s="2" t="n">
         <v>2300</v>
       </c>
+      <c r="G127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4016,6 +4148,7 @@
       <c r="F128" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="G128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4044,6 +4177,7 @@
       <c r="F129" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="G129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4072,6 +4206,7 @@
       <c r="F130" s="2" t="n">
         <v>375</v>
       </c>
+      <c r="G130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4100,6 +4235,7 @@
       <c r="F131" s="2" t="n">
         <v>225</v>
       </c>
+      <c r="G131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4128,6 +4264,7 @@
       <c r="F132" s="2" t="n">
         <v>225</v>
       </c>
+      <c r="G132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4156,6 +4293,7 @@
       <c r="F133" s="2" t="n">
         <v>420</v>
       </c>
+      <c r="G133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4184,6 +4322,7 @@
       <c r="F134" s="2" t="n">
         <v>450</v>
       </c>
+      <c r="G134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4212,6 +4351,7 @@
       <c r="F135" s="2" t="n">
         <v>125</v>
       </c>
+      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4240,6 +4380,7 @@
       <c r="F136" s="2" t="n">
         <v>555</v>
       </c>
+      <c r="G136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4268,6 +4409,7 @@
       <c r="F137" s="2" t="n">
         <v>69</v>
       </c>
+      <c r="G137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4296,6 +4438,7 @@
       <c r="F138" s="2" t="n">
         <v>90</v>
       </c>
+      <c r="G138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4324,6 +4467,7 @@
       <c r="F139" s="2" t="n">
         <v>81</v>
       </c>
+      <c r="G139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4352,6 +4496,7 @@
       <c r="F140" s="2" t="n">
         <v>13.5</v>
       </c>
+      <c r="G140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4380,6 +4525,7 @@
       <c r="F141" s="2" t="n">
         <v>29.5</v>
       </c>
+      <c r="G141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4408,6 +4554,7 @@
       <c r="F142" s="2" t="n">
         <v>28.5</v>
       </c>
+      <c r="G142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4436,6 +4583,7 @@
       <c r="F143" s="2" t="n">
         <v>105</v>
       </c>
+      <c r="G143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4464,6 +4612,7 @@
       <c r="F144" s="2" t="n">
         <v>240</v>
       </c>
+      <c r="G144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4492,6 +4641,7 @@
       <c r="F145" s="2" t="n">
         <v>850</v>
       </c>
+      <c r="G145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -4520,6 +4670,7 @@
       <c r="F146" s="2" t="n">
         <v>2300</v>
       </c>
+      <c r="G146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4548,6 +4699,7 @@
       <c r="F147" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="G147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -4576,6 +4728,7 @@
       <c r="F148" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="G148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -4604,6 +4757,7 @@
       <c r="F149" s="2" t="n">
         <v>375</v>
       </c>
+      <c r="G149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -4632,6 +4786,7 @@
       <c r="F150" s="2" t="n">
         <v>225</v>
       </c>
+      <c r="G150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -4660,6 +4815,7 @@
       <c r="F151" s="2" t="n">
         <v>225</v>
       </c>
+      <c r="G151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -4688,6 +4844,7 @@
       <c r="F152" s="2" t="n">
         <v>420</v>
       </c>
+      <c r="G152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -4716,6 +4873,7 @@
       <c r="F153" s="2" t="n">
         <v>450</v>
       </c>
+      <c r="G153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -4744,6 +4902,7 @@
       <c r="F154" s="2" t="n">
         <v>125</v>
       </c>
+      <c r="G154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -4772,6 +4931,7 @@
       <c r="F155" s="2" t="n">
         <v>555</v>
       </c>
+      <c r="G155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -4800,6 +4960,7 @@
       <c r="F156" s="2" t="n">
         <v>69</v>
       </c>
+      <c r="G156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -4828,6 +4989,7 @@
       <c r="F157" s="2" t="n">
         <v>90</v>
       </c>
+      <c r="G157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -4856,6 +5018,7 @@
       <c r="F158" s="2" t="n">
         <v>81</v>
       </c>
+      <c r="G158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -4884,6 +5047,7 @@
       <c r="F159" s="2" t="n">
         <v>13.5</v>
       </c>
+      <c r="G159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -4912,6 +5076,7 @@
       <c r="F160" s="2" t="n">
         <v>29.5</v>
       </c>
+      <c r="G160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -4940,6 +5105,7 @@
       <c r="F161" s="2" t="n">
         <v>28.5</v>
       </c>
+      <c r="G161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -4968,6 +5134,7 @@
       <c r="F162" s="2" t="n">
         <v>105</v>
       </c>
+      <c r="G162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -4996,6 +5163,7 @@
       <c r="F163" s="2" t="n">
         <v>240</v>
       </c>
+      <c r="G163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -5024,6 +5192,7 @@
       <c r="F164" s="2" t="n">
         <v>850</v>
       </c>
+      <c r="G164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -5052,6 +5221,7 @@
       <c r="F165" s="2" t="n">
         <v>2300</v>
       </c>
+      <c r="G165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -5080,6 +5250,7 @@
       <c r="F166" s="2" t="n">
         <v>3534</v>
       </c>
+      <c r="G166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -5108,6 +5279,7 @@
       <c r="F167" s="2" t="n">
         <v>3534</v>
       </c>
+      <c r="G167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -5136,6 +5308,7 @@
       <c r="F168" s="2" t="n">
         <v>3534</v>
       </c>
+      <c r="G168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -5164,6 +5337,7 @@
       <c r="F169" s="2" t="n">
         <v>2584</v>
       </c>
+      <c r="G169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -5192,6 +5366,7 @@
       <c r="F170" s="2" t="n">
         <v>725</v>
       </c>
+      <c r="G170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -5220,6 +5395,7 @@
       <c r="F171" s="2" t="n">
         <v>725</v>
       </c>
+      <c r="G171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -5248,6 +5424,7 @@
       <c r="F172" s="2" t="n">
         <v>725</v>
       </c>
+      <c r="G172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -5276,6 +5453,7 @@
       <c r="F173" s="2" t="n">
         <v>725</v>
       </c>
+      <c r="G173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -5304,6 +5482,7 @@
       <c r="F174" s="2" t="n">
         <v>2703</v>
       </c>
+      <c r="G174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -5332,6 +5511,7 @@
       <c r="F175" s="2" t="n">
         <v>1025</v>
       </c>
+      <c r="G175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -5360,6 +5540,7 @@
       <c r="F176" s="2" t="n">
         <v>1025</v>
       </c>
+      <c r="G176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -5388,6 +5569,7 @@
       <c r="F177" s="2" t="n">
         <v>1025</v>
       </c>
+      <c r="G177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -5416,6 +5598,7 @@
       <c r="F178" s="2" t="n">
         <v>1025</v>
       </c>
+      <c r="G178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -5444,6 +5627,7 @@
       <c r="F179" s="2" t="n">
         <v>2470</v>
       </c>
+      <c r="G179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -5472,6 +5656,7 @@
       <c r="F180" s="2" t="n">
         <v>825</v>
       </c>
+      <c r="G180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -5500,6 +5685,7 @@
       <c r="F181" s="2" t="n">
         <v>825</v>
       </c>
+      <c r="G181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -5528,6 +5714,7 @@
       <c r="F182" s="2" t="n">
         <v>825</v>
       </c>
+      <c r="G182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -5556,6 +5743,7 @@
       <c r="F183" s="2" t="n">
         <v>825</v>
       </c>
+      <c r="G183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -5584,6 +5772,7 @@
       <c r="F184" s="2" t="n">
         <v>547</v>
       </c>
+      <c r="G184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -5612,6 +5801,7 @@
       <c r="F185" s="2" t="n">
         <v>547</v>
       </c>
+      <c r="G185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -5640,6 +5830,7 @@
       <c r="F186" s="2" t="n">
         <v>547</v>
       </c>
+      <c r="G186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -5668,6 +5859,7 @@
       <c r="F187" s="2" t="n">
         <v>547</v>
       </c>
+      <c r="G187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -5696,6 +5888,7 @@
       <c r="F188" s="2" t="n">
         <v>3210</v>
       </c>
+      <c r="G188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -5724,6 +5917,7 @@
       <c r="F189" s="2" t="n">
         <v>8567</v>
       </c>
+      <c r="G189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -5752,6 +5946,7 @@
       <c r="F190" s="2" t="n">
         <v>501</v>
       </c>
+      <c r="G190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -5780,6 +5975,7 @@
       <c r="F191" s="2" t="n">
         <v>8926</v>
       </c>
+      <c r="G191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -5808,6 +6004,7 @@
       <c r="F192" s="2" t="n">
         <v>735</v>
       </c>
+      <c r="G192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -5836,6 +6033,7 @@
       <c r="F193" s="2" t="n">
         <v>9330</v>
       </c>
+      <c r="G193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -5864,6 +6062,7 @@
       <c r="F194" s="2" t="n">
         <v>526</v>
       </c>
+      <c r="G194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -5892,6 +6091,7 @@
       <c r="F195" s="2" t="n">
         <v>430</v>
       </c>
+      <c r="G195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -5919,6 +6119,40 @@
       </c>
       <c r="F196" s="2" t="n">
         <v>300</v>
+      </c>
+      <c r="G196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Ishani Ridge (Century Complete)</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Plan Pricing</t>
+        </is>
+      </c>
+      <c r="C197" s="1" t="n">
+        <v>46153</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="F197" s="2" t="n">
+        <v>2765</v>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Price reduced from contract approved by Tony</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add missing contracts: Tri Pointe (Agave Ridge, Edgewood), Bluffs I/II + Arroyo concrete, Woodside Meridian/Estrella/Luna, Other Builders (AMH, Blue Heron, Pinnacle); Duplex concrete moved to signed 6/1/2026 contract
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D6wjrb1spFgY1HgqZrWwPC
</commit_message>
<xml_diff>
--- a/CenturyCommunitiesContracts1.xlsx
+++ b/CenturyCommunitiesContracts1.xlsx
@@ -418,16 +418,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G197"/>
+  <dimension ref="A1:G233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6155,6 +6155,1050 @@
         </is>
       </c>
     </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C198" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>1663</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="n">
+        <v>11550</v>
+      </c>
+      <c r="G198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C199" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>1663</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>BED0035 - Bedroom 3/Bath Elevation B</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="n">
+        <v>439</v>
+      </c>
+      <c r="G199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C200" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>1663</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>BED0036 - Bedroom 3/Bath Elevation C</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="n">
+        <v>439</v>
+      </c>
+      <c r="G200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C201" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>1663</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="n">
+        <v>437</v>
+      </c>
+      <c r="G201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C202" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>1663</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>CP0207 - Patio Cover A - Elevation B</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="n">
+        <v>428</v>
+      </c>
+      <c r="G202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C203" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>1663</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>CP0208 - Patio Cover A - Elevation C</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="n">
+        <v>663</v>
+      </c>
+      <c r="G203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C204" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>1742</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="n">
+        <v>11684</v>
+      </c>
+      <c r="G204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C205" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>1742</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="n">
+        <v>374</v>
+      </c>
+      <c r="G205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C206" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>1742</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>CP0207 - Patio Cover A - Elevation B</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="n">
+        <v>1277</v>
+      </c>
+      <c r="G206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C207" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>1742</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>CP0208 - Patio Cover A - Elevation C</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="n">
+        <v>1277</v>
+      </c>
+      <c r="G207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C208" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>1831</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="n">
+        <v>12346</v>
+      </c>
+      <c r="G208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C209" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>1831</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="n">
+        <v>692</v>
+      </c>
+      <c r="G209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C210" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>1831</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>CP0207 - Patio Cover A - Elevation B</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="n">
+        <v>714</v>
+      </c>
+      <c r="G210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C211" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>1831</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>CP0208 - Patio Cover A - Elevation C</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="n">
+        <v>714</v>
+      </c>
+      <c r="G211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C212" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>1831</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>BED0040 - Bedroom 4/Bath</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="n">
+        <v>570</v>
+      </c>
+      <c r="G212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C213" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="n">
+        <v>12646</v>
+      </c>
+      <c r="G213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C214" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="n">
+        <v>720</v>
+      </c>
+      <c r="G214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C215" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>CP0207 - Patio Cover A - Elevation B</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="n">
+        <v>720</v>
+      </c>
+      <c r="G215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C216" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>CP0208 - Patio Cover A - Elevation C</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="n">
+        <v>720</v>
+      </c>
+      <c r="G216" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C217" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>CAS0007 - Guest Quarters w/Direct Access - A</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="n">
+        <v>4368</v>
+      </c>
+      <c r="G217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C218" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>CAS0008 - Guest Quarters w/Direct Access - B</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="n">
+        <v>4368</v>
+      </c>
+      <c r="G218" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C219" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>CAS0009 - Guest Quarters w/Direct Access - C</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="n">
+        <v>4368</v>
+      </c>
+      <c r="G219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C220" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>2230</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="n">
+        <v>14023</v>
+      </c>
+      <c r="G220" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C221" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>2230</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F221" s="2" t="n">
+        <v>559</v>
+      </c>
+      <c r="G221" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C222" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>2230</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>CP0207 - Patio Cover A - Elevation B</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="n">
+        <v>619</v>
+      </c>
+      <c r="G222" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C223" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>2230</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>CP0208 - Patio Cover A - Elevation C</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="n">
+        <v>657</v>
+      </c>
+      <c r="G223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C224" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="n">
+        <v>14913</v>
+      </c>
+      <c r="G224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C225" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="n">
+        <v>720</v>
+      </c>
+      <c r="G225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C226" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>CP0207 - Patio Cover A - Elevation B</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="n">
+        <v>720</v>
+      </c>
+      <c r="G226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C227" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>CP0208 - Patio Cover A - Elevation C</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="n">
+        <v>720</v>
+      </c>
+      <c r="G227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C228" s="1" t="n">
+        <v>45839</v>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Beverly</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F228" s="2" t="n">
+        <v>5273</v>
+      </c>
+      <c r="G228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C229" s="1" t="n">
+        <v>45839</v>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Captiva</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="n">
+        <v>5659</v>
+      </c>
+      <c r="G229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C230" s="1" t="n">
+        <v>45839</v>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Delray</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F230" s="2" t="n">
+        <v>5955</v>
+      </c>
+      <c r="G230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C231" s="1" t="n">
+        <v>45992</v>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Beverly</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F231" s="2" t="n">
+        <v>4925</v>
+      </c>
+      <c r="G231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C232" s="1" t="n">
+        <v>45992</v>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Captiva</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F232" s="2" t="n">
+        <v>5286</v>
+      </c>
+      <c r="G232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C233" s="1" t="n">
+        <v>45992</v>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Delray</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F233" s="2" t="n">
+        <v>5562</v>
+      </c>
+      <c r="G233" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Century Edgeview Estates pavers pricing (PPS 5002087, eff 11/1/26)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D6wjrb1spFgY1HgqZrWwPC
</commit_message>
<xml_diff>
--- a/CenturyCommunitiesContracts1.xlsx
+++ b/CenturyCommunitiesContracts1.xlsx
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,10 +49,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G233"/>
+  <dimension ref="A1:G236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -478,7 +479,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="3" t="n">
         <v>45505</v>
       </c>
       <c r="D2" t="inlineStr">
@@ -494,7 +495,6 @@
       <c r="F2" s="2" t="n">
         <v>6450</v>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -507,7 +507,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="3" t="n">
         <v>45505</v>
       </c>
       <c r="D3" t="inlineStr">
@@ -523,7 +523,6 @@
       <c r="F3" s="2" t="n">
         <v>6788</v>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -536,7 +535,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="3" t="n">
         <v>45505</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -552,7 +551,6 @@
       <c r="F4" s="2" t="n">
         <v>6788</v>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -565,7 +563,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="C5" s="3" t="n">
         <v>45505</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -581,7 +579,6 @@
       <c r="F5" s="2" t="n">
         <v>6791</v>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -594,7 +591,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -610,7 +607,6 @@
       <c r="F6" s="2" t="n">
         <v>6704</v>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -623,7 +619,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="C7" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -639,7 +635,6 @@
       <c r="F7" s="2" t="n">
         <v>555</v>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -652,7 +647,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="C8" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -668,7 +663,6 @@
       <c r="F8" s="2" t="n">
         <v>6596</v>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -681,7 +675,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C9" s="1" t="n">
+      <c r="C9" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -697,7 +691,6 @@
       <c r="F9" s="2" t="n">
         <v>580</v>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -710,7 +703,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -726,7 +719,6 @@
       <c r="F10" s="2" t="n">
         <v>7112</v>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -739,7 +731,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="C11" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D11" t="inlineStr">
@@ -755,7 +747,6 @@
       <c r="F11" s="2" t="n">
         <v>580</v>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -768,7 +759,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C12" s="1" t="n">
+      <c r="C12" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D12" t="inlineStr">
@@ -784,7 +775,6 @@
       <c r="F12" s="2" t="n">
         <v>6966</v>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -797,7 +787,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C13" s="1" t="n">
+      <c r="C13" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D13" t="inlineStr">
@@ -813,7 +803,6 @@
       <c r="F13" s="2" t="n">
         <v>581</v>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -826,7 +815,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C14" s="1" t="n">
+      <c r="C14" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -842,7 +831,6 @@
       <c r="F14" s="2" t="n">
         <v>581</v>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -855,7 +843,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C15" s="1" t="n">
+      <c r="C15" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D15" t="inlineStr">
@@ -871,7 +859,6 @@
       <c r="F15" s="2" t="n">
         <v>581</v>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -884,7 +871,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C16" s="1" t="n">
+      <c r="C16" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D16" t="inlineStr">
@@ -900,7 +887,6 @@
       <c r="F16" s="2" t="n">
         <v>581</v>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -913,7 +899,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C17" s="1" t="n">
+      <c r="C17" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D17" t="inlineStr">
@@ -929,7 +915,6 @@
       <c r="F17" s="2" t="n">
         <v>581</v>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -942,7 +927,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="C18" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D18" t="inlineStr">
@@ -958,7 +943,6 @@
       <c r="F18" s="2" t="n">
         <v>7162</v>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -971,7 +955,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C19" s="1" t="n">
+      <c r="C19" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D19" t="inlineStr">
@@ -987,7 +971,6 @@
       <c r="F19" s="2" t="n">
         <v>579</v>
       </c>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1000,7 +983,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C20" s="1" t="n">
+      <c r="C20" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D20" t="inlineStr">
@@ -1016,7 +999,6 @@
       <c r="F20" s="2" t="n">
         <v>579</v>
       </c>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1029,7 +1011,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C21" s="1" t="n">
+      <c r="C21" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D21" t="inlineStr">
@@ -1045,7 +1027,6 @@
       <c r="F21" s="2" t="n">
         <v>579</v>
       </c>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1058,7 +1039,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C22" s="1" t="n">
+      <c r="C22" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D22" t="inlineStr">
@@ -1074,7 +1055,6 @@
       <c r="F22" s="2" t="n">
         <v>579</v>
       </c>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1087,7 +1067,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C23" s="1" t="n">
+      <c r="C23" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D23" t="inlineStr">
@@ -1103,7 +1083,6 @@
       <c r="F23" s="2" t="n">
         <v>579</v>
       </c>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1116,7 +1095,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C24" s="1" t="n">
+      <c r="C24" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D24" t="inlineStr">
@@ -1132,7 +1111,6 @@
       <c r="F24" s="2" t="n">
         <v>7096</v>
       </c>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1145,7 +1123,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C25" s="1" t="n">
+      <c r="C25" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D25" t="inlineStr">
@@ -1161,7 +1139,6 @@
       <c r="F25" s="2" t="n">
         <v>549</v>
       </c>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1174,7 +1151,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C26" s="1" t="n">
+      <c r="C26" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D26" t="inlineStr">
@@ -1190,7 +1167,6 @@
       <c r="F26" s="2" t="n">
         <v>549</v>
       </c>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1203,7 +1179,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C27" s="1" t="n">
+      <c r="C27" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D27" t="inlineStr">
@@ -1219,7 +1195,6 @@
       <c r="F27" s="2" t="n">
         <v>549</v>
       </c>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1232,7 +1207,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C28" s="1" t="n">
+      <c r="C28" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D28" t="inlineStr">
@@ -1248,7 +1223,6 @@
       <c r="F28" s="2" t="n">
         <v>549</v>
       </c>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1261,7 +1235,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C29" s="1" t="n">
+      <c r="C29" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D29" t="inlineStr">
@@ -1277,7 +1251,6 @@
       <c r="F29" s="2" t="n">
         <v>7802</v>
       </c>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1290,7 +1263,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C30" s="1" t="n">
+      <c r="C30" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D30" t="inlineStr">
@@ -1306,7 +1279,6 @@
       <c r="F30" s="2" t="n">
         <v>588</v>
       </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1319,7 +1291,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C31" s="1" t="n">
+      <c r="C31" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D31" t="inlineStr">
@@ -1335,7 +1307,6 @@
       <c r="F31" s="2" t="n">
         <v>588</v>
       </c>
-      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1348,7 +1319,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C32" s="1" t="n">
+      <c r="C32" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D32" t="inlineStr">
@@ -1364,7 +1335,6 @@
       <c r="F32" s="2" t="n">
         <v>588</v>
       </c>
-      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1377,7 +1347,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C33" s="1" t="n">
+      <c r="C33" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D33" t="inlineStr">
@@ -1393,7 +1363,6 @@
       <c r="F33" s="2" t="n">
         <v>549</v>
       </c>
-      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1406,7 +1375,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C34" s="1" t="n">
+      <c r="C34" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D34" t="inlineStr">
@@ -1422,7 +1391,6 @@
       <c r="F34" s="2" t="n">
         <v>588</v>
       </c>
-      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1435,7 +1403,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C35" s="1" t="n">
+      <c r="C35" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D35" t="inlineStr">
@@ -1451,7 +1419,6 @@
       <c r="F35" s="2" t="n">
         <v>7270</v>
       </c>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1464,7 +1431,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C36" s="1" t="n">
+      <c r="C36" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D36" t="inlineStr">
@@ -1480,7 +1447,6 @@
       <c r="F36" s="2" t="n">
         <v>702</v>
       </c>
-      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1493,7 +1459,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C37" s="1" t="n">
+      <c r="C37" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D37" t="inlineStr">
@@ -1509,7 +1475,6 @@
       <c r="F37" s="2" t="n">
         <v>702</v>
       </c>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1522,7 +1487,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C38" s="1" t="n">
+      <c r="C38" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D38" t="inlineStr">
@@ -1538,7 +1503,6 @@
       <c r="F38" s="2" t="n">
         <v>702</v>
       </c>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1551,7 +1515,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C39" s="1" t="n">
+      <c r="C39" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D39" t="inlineStr">
@@ -1567,7 +1531,6 @@
       <c r="F39" s="2" t="n">
         <v>702</v>
       </c>
-      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1580,7 +1543,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C40" s="1" t="n">
+      <c r="C40" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D40" t="inlineStr">
@@ -1596,7 +1559,6 @@
       <c r="F40" s="2" t="n">
         <v>702</v>
       </c>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1609,7 +1571,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C41" s="1" t="n">
+      <c r="C41" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D41" t="inlineStr">
@@ -1625,7 +1587,6 @@
       <c r="F41" s="2" t="n">
         <v>7450</v>
       </c>
-      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1638,7 +1599,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C42" s="1" t="n">
+      <c r="C42" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D42" t="inlineStr">
@@ -1654,7 +1615,6 @@
       <c r="F42" s="2" t="n">
         <v>513</v>
       </c>
-      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1667,7 +1627,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C43" s="1" t="n">
+      <c r="C43" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D43" t="inlineStr">
@@ -1683,7 +1643,6 @@
       <c r="F43" s="2" t="n">
         <v>513</v>
       </c>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1696,7 +1655,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C44" s="1" t="n">
+      <c r="C44" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D44" t="inlineStr">
@@ -1712,7 +1671,6 @@
       <c r="F44" s="2" t="n">
         <v>513</v>
       </c>
-      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1725,7 +1683,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C45" s="1" t="n">
+      <c r="C45" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D45" t="inlineStr">
@@ -1741,7 +1699,6 @@
       <c r="F45" s="2" t="n">
         <v>513</v>
       </c>
-      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1754,7 +1711,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C46" s="1" t="n">
+      <c r="C46" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D46" t="inlineStr">
@@ -1770,7 +1727,6 @@
       <c r="F46" s="2" t="n">
         <v>513</v>
       </c>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1783,7 +1739,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C47" s="1" t="n">
+      <c r="C47" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D47" t="inlineStr">
@@ -1799,7 +1755,6 @@
       <c r="F47" s="2" t="n">
         <v>7713</v>
       </c>
-      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1812,7 +1767,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C48" s="1" t="n">
+      <c r="C48" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D48" t="inlineStr">
@@ -1828,7 +1783,6 @@
       <c r="F48" s="2" t="n">
         <v>504</v>
       </c>
-      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1841,7 +1795,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C49" s="1" t="n">
+      <c r="C49" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D49" t="inlineStr">
@@ -1857,7 +1811,6 @@
       <c r="F49" s="2" t="n">
         <v>504</v>
       </c>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1870,7 +1823,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C50" s="1" t="n">
+      <c r="C50" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D50" t="inlineStr">
@@ -1886,7 +1839,6 @@
       <c r="F50" s="2" t="n">
         <v>504</v>
       </c>
-      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1899,7 +1851,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C51" s="1" t="n">
+      <c r="C51" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D51" t="inlineStr">
@@ -1915,7 +1867,6 @@
       <c r="F51" s="2" t="n">
         <v>504</v>
       </c>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1928,7 +1879,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C52" s="1" t="n">
+      <c r="C52" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D52" t="inlineStr">
@@ -1944,7 +1895,6 @@
       <c r="F52" s="2" t="n">
         <v>504</v>
       </c>
-      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1957,7 +1907,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C53" s="1" t="n">
+      <c r="C53" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D53" t="inlineStr">
@@ -1973,7 +1923,6 @@
       <c r="F53" s="2" t="n">
         <v>6295</v>
       </c>
-      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1986,7 +1935,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C54" s="1" t="n">
+      <c r="C54" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D54" t="inlineStr">
@@ -2002,7 +1951,6 @@
       <c r="F54" s="2" t="n">
         <v>6665</v>
       </c>
-      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2015,7 +1963,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C55" s="1" t="n">
+      <c r="C55" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D55" t="inlineStr">
@@ -2031,7 +1979,6 @@
       <c r="F55" s="2" t="n">
         <v>7324</v>
       </c>
-      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2044,7 +1991,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C56" s="1" t="n">
+      <c r="C56" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D56" t="inlineStr">
@@ -2060,7 +2007,6 @@
       <c r="F56" s="2" t="n">
         <v>6434</v>
       </c>
-      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2073,7 +2019,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C57" s="1" t="n">
+      <c r="C57" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D57" t="inlineStr">
@@ -2089,7 +2035,6 @@
       <c r="F57" s="2" t="n">
         <v>541</v>
       </c>
-      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2102,7 +2047,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C58" s="1" t="n">
+      <c r="C58" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D58" t="inlineStr">
@@ -2118,7 +2063,6 @@
       <c r="F58" s="2" t="n">
         <v>6755</v>
       </c>
-      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2131,7 +2075,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C59" s="1" t="n">
+      <c r="C59" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D59" t="inlineStr">
@@ -2147,7 +2091,6 @@
       <c r="F59" s="2" t="n">
         <v>541</v>
       </c>
-      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2160,7 +2103,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C60" s="1" t="n">
+      <c r="C60" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D60" t="inlineStr">
@@ -2176,7 +2119,6 @@
       <c r="F60" s="2" t="n">
         <v>6989</v>
       </c>
-      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2189,7 +2131,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C61" s="1" t="n">
+      <c r="C61" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D61" t="inlineStr">
@@ -2205,7 +2147,6 @@
       <c r="F61" s="2" t="n">
         <v>525</v>
       </c>
-      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2218,7 +2159,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C62" s="1" t="n">
+      <c r="C62" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D62" t="inlineStr">
@@ -2234,7 +2175,6 @@
       <c r="F62" s="2" t="n">
         <v>6630</v>
       </c>
-      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2247,7 +2187,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C63" s="1" t="n">
+      <c r="C63" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D63" t="inlineStr">
@@ -2263,7 +2203,6 @@
       <c r="F63" s="2" t="n">
         <v>350</v>
       </c>
-      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2276,7 +2215,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C64" s="1" t="n">
+      <c r="C64" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D64" t="inlineStr">
@@ -2292,7 +2231,6 @@
       <c r="F64" s="2" t="n">
         <v>7194</v>
       </c>
-      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2305,7 +2243,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C65" s="1" t="n">
+      <c r="C65" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D65" t="inlineStr">
@@ -2321,7 +2259,6 @@
       <c r="F65" s="2" t="n">
         <v>350</v>
       </c>
-      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2334,7 +2271,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C66" s="1" t="n">
+      <c r="C66" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D66" t="inlineStr">
@@ -2350,7 +2287,6 @@
       <c r="F66" s="2" t="n">
         <v>7575</v>
       </c>
-      <c r="G66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2363,7 +2299,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C67" s="1" t="n">
+      <c r="C67" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D67" t="inlineStr">
@@ -2379,7 +2315,6 @@
       <c r="F67" s="2" t="n">
         <v>350</v>
       </c>
-      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2392,7 +2327,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C68" s="1" t="n">
+      <c r="C68" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D68" t="inlineStr">
@@ -2408,7 +2343,6 @@
       <c r="F68" s="2" t="n">
         <v>3012</v>
       </c>
-      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2421,7 +2355,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C69" s="1" t="n">
+      <c r="C69" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D69" t="inlineStr">
@@ -2437,7 +2371,6 @@
       <c r="F69" s="2" t="n">
         <v>4216</v>
       </c>
-      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2450,7 +2383,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C70" s="1" t="n">
+      <c r="C70" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D70" t="inlineStr">
@@ -2466,7 +2399,6 @@
       <c r="F70" s="2" t="n">
         <v>1804</v>
       </c>
-      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2479,7 +2411,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C71" s="1" t="n">
+      <c r="C71" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D71" t="inlineStr">
@@ -2495,7 +2427,6 @@
       <c r="F71" s="2" t="n">
         <v>720</v>
       </c>
-      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2508,7 +2439,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C72" s="1" t="n">
+      <c r="C72" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D72" t="inlineStr">
@@ -2524,7 +2455,6 @@
       <c r="F72" s="2" t="n">
         <v>960</v>
       </c>
-      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2537,7 +2467,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C73" s="1" t="n">
+      <c r="C73" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D73" t="inlineStr">
@@ -2553,7 +2483,6 @@
       <c r="F73" s="2" t="n">
         <v>480</v>
       </c>
-      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2566,7 +2495,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C74" s="1" t="n">
+      <c r="C74" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D74" t="inlineStr">
@@ -2582,7 +2511,6 @@
       <c r="F74" s="2" t="n">
         <v>660</v>
       </c>
-      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2595,7 +2523,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C75" s="1" t="n">
+      <c r="C75" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D75" t="inlineStr">
@@ -2611,7 +2539,6 @@
       <c r="F75" s="2" t="n">
         <v>960</v>
       </c>
-      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2624,7 +2551,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C76" s="1" t="n">
+      <c r="C76" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D76" t="inlineStr">
@@ -2640,7 +2567,6 @@
       <c r="F76" s="2" t="n">
         <v>480</v>
       </c>
-      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2653,7 +2579,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C77" s="1" t="n">
+      <c r="C77" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D77" t="inlineStr">
@@ -2669,7 +2595,6 @@
       <c r="F77" s="2" t="n">
         <v>2259</v>
       </c>
-      <c r="G77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2682,7 +2607,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C78" s="1" t="n">
+      <c r="C78" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D78" t="inlineStr">
@@ -2698,7 +2623,6 @@
       <c r="F78" s="2" t="n">
         <v>3162</v>
       </c>
-      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2711,7 +2635,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C79" s="1" t="n">
+      <c r="C79" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D79" t="inlineStr">
@@ -2727,7 +2651,6 @@
       <c r="F79" s="2" t="n">
         <v>1353</v>
       </c>
-      <c r="G79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2740,7 +2663,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C80" s="1" t="n">
+      <c r="C80" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D80" t="inlineStr">
@@ -2756,7 +2679,6 @@
       <c r="F80" s="2" t="n">
         <v>540</v>
       </c>
-      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2769,7 +2691,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C81" s="1" t="n">
+      <c r="C81" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D81" t="inlineStr">
@@ -2785,7 +2707,6 @@
       <c r="F81" s="2" t="n">
         <v>720</v>
       </c>
-      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2798,7 +2719,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C82" s="1" t="n">
+      <c r="C82" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D82" t="inlineStr">
@@ -2814,7 +2735,6 @@
       <c r="F82" s="2" t="n">
         <v>360</v>
       </c>
-      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2827,7 +2747,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C83" s="1" t="n">
+      <c r="C83" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D83" t="inlineStr">
@@ -2843,7 +2763,6 @@
       <c r="F83" s="2" t="n">
         <v>495</v>
       </c>
-      <c r="G83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2856,7 +2775,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C84" s="1" t="n">
+      <c r="C84" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D84" t="inlineStr">
@@ -2872,7 +2791,6 @@
       <c r="F84" s="2" t="n">
         <v>720</v>
       </c>
-      <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2885,7 +2803,7 @@
           <t>Drop Garage</t>
         </is>
       </c>
-      <c r="C85" s="1" t="n">
+      <c r="C85" s="3" t="n">
         <v>45397</v>
       </c>
       <c r="D85" t="inlineStr">
@@ -2901,7 +2819,6 @@
       <c r="F85" s="2" t="n">
         <v>360</v>
       </c>
-      <c r="G85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2914,7 +2831,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C86" s="1" t="n">
+      <c r="C86" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D86" t="inlineStr">
@@ -2930,7 +2847,6 @@
       <c r="F86" s="2" t="n">
         <v>5714</v>
       </c>
-      <c r="G86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2943,7 +2859,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C87" s="1" t="n">
+      <c r="C87" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D87" t="inlineStr">
@@ -2959,7 +2875,6 @@
       <c r="F87" s="2" t="n">
         <v>6012</v>
       </c>
-      <c r="G87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2972,7 +2887,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C88" s="1" t="n">
+      <c r="C88" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D88" t="inlineStr">
@@ -2988,7 +2903,6 @@
       <c r="F88" s="2" t="n">
         <v>6012</v>
       </c>
-      <c r="G88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3001,7 +2915,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C89" s="1" t="n">
+      <c r="C89" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D89" t="inlineStr">
@@ -3017,7 +2931,6 @@
       <c r="F89" s="2" t="n">
         <v>6016</v>
       </c>
-      <c r="G89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3030,7 +2943,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C90" s="1" t="n">
+      <c r="C90" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D90" t="inlineStr">
@@ -3046,7 +2959,6 @@
       <c r="F90" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3059,7 +2971,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C91" s="1" t="n">
+      <c r="C91" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D91" t="inlineStr">
@@ -3075,7 +2987,6 @@
       <c r="F91" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3088,7 +2999,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C92" s="1" t="n">
+      <c r="C92" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D92" t="inlineStr">
@@ -3104,7 +3015,6 @@
       <c r="F92" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3117,7 +3027,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C93" s="1" t="n">
+      <c r="C93" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D93" t="inlineStr">
@@ -3133,7 +3043,6 @@
       <c r="F93" s="2" t="n">
         <v>225</v>
       </c>
-      <c r="G93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3146,7 +3055,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C94" s="1" t="n">
+      <c r="C94" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D94" t="inlineStr">
@@ -3162,7 +3071,6 @@
       <c r="F94" s="2" t="n">
         <v>225</v>
       </c>
-      <c r="G94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3175,7 +3083,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C95" s="1" t="n">
+      <c r="C95" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D95" t="inlineStr">
@@ -3191,7 +3099,6 @@
       <c r="F95" s="2" t="n">
         <v>420</v>
       </c>
-      <c r="G95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3204,7 +3111,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C96" s="1" t="n">
+      <c r="C96" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D96" t="inlineStr">
@@ -3220,7 +3127,6 @@
       <c r="F96" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="G96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3233,7 +3139,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C97" s="1" t="n">
+      <c r="C97" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D97" t="inlineStr">
@@ -3249,7 +3155,6 @@
       <c r="F97" s="2" t="n">
         <v>125</v>
       </c>
-      <c r="G97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3262,7 +3167,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C98" s="1" t="n">
+      <c r="C98" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D98" t="inlineStr">
@@ -3278,7 +3183,6 @@
       <c r="F98" s="2" t="n">
         <v>555</v>
       </c>
-      <c r="G98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3291,7 +3195,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C99" s="1" t="n">
+      <c r="C99" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D99" t="inlineStr">
@@ -3307,7 +3211,6 @@
       <c r="F99" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="G99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3320,7 +3223,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C100" s="1" t="n">
+      <c r="C100" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D100" t="inlineStr">
@@ -3336,7 +3239,6 @@
       <c r="F100" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="G100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3349,7 +3251,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C101" s="1" t="n">
+      <c r="C101" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D101" t="inlineStr">
@@ -3365,7 +3267,6 @@
       <c r="F101" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="G101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3378,7 +3279,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C102" s="1" t="n">
+      <c r="C102" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D102" t="inlineStr">
@@ -3394,7 +3295,6 @@
       <c r="F102" s="2" t="n">
         <v>13.5</v>
       </c>
-      <c r="G102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3407,7 +3307,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C103" s="1" t="n">
+      <c r="C103" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D103" t="inlineStr">
@@ -3423,7 +3323,6 @@
       <c r="F103" s="2" t="n">
         <v>29.5</v>
       </c>
-      <c r="G103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3436,7 +3335,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C104" s="1" t="n">
+      <c r="C104" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D104" t="inlineStr">
@@ -3452,7 +3351,6 @@
       <c r="F104" s="2" t="n">
         <v>28.5</v>
       </c>
-      <c r="G104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3465,7 +3363,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C105" s="1" t="n">
+      <c r="C105" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D105" t="inlineStr">
@@ -3481,7 +3379,6 @@
       <c r="F105" s="2" t="n">
         <v>105</v>
       </c>
-      <c r="G105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3494,7 +3391,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C106" s="1" t="n">
+      <c r="C106" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D106" t="inlineStr">
@@ -3510,7 +3407,6 @@
       <c r="F106" s="2" t="n">
         <v>240</v>
       </c>
-      <c r="G106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3523,7 +3419,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C107" s="1" t="n">
+      <c r="C107" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D107" t="inlineStr">
@@ -3539,7 +3435,6 @@
       <c r="F107" s="2" t="n">
         <v>850</v>
       </c>
-      <c r="G107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3552,7 +3447,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C108" s="1" t="n">
+      <c r="C108" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D108" t="inlineStr">
@@ -3568,7 +3463,6 @@
       <c r="F108" s="2" t="n">
         <v>2300</v>
       </c>
-      <c r="G108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3581,7 +3475,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C109" s="1" t="n">
+      <c r="C109" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D109" t="inlineStr">
@@ -3597,7 +3491,6 @@
       <c r="F109" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3610,7 +3503,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C110" s="1" t="n">
+      <c r="C110" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D110" t="inlineStr">
@@ -3626,7 +3519,6 @@
       <c r="F110" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3639,7 +3531,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C111" s="1" t="n">
+      <c r="C111" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D111" t="inlineStr">
@@ -3655,7 +3547,6 @@
       <c r="F111" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="G111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3668,7 +3559,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C112" s="1" t="n">
+      <c r="C112" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D112" t="inlineStr">
@@ -3684,7 +3575,6 @@
       <c r="F112" s="2" t="n">
         <v>225</v>
       </c>
-      <c r="G112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3697,7 +3587,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C113" s="1" t="n">
+      <c r="C113" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D113" t="inlineStr">
@@ -3713,7 +3603,6 @@
       <c r="F113" s="2" t="n">
         <v>225</v>
       </c>
-      <c r="G113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3726,7 +3615,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C114" s="1" t="n">
+      <c r="C114" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D114" t="inlineStr">
@@ -3742,7 +3631,6 @@
       <c r="F114" s="2" t="n">
         <v>420</v>
       </c>
-      <c r="G114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3755,7 +3643,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C115" s="1" t="n">
+      <c r="C115" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D115" t="inlineStr">
@@ -3771,7 +3659,6 @@
       <c r="F115" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="G115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3784,7 +3671,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C116" s="1" t="n">
+      <c r="C116" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D116" t="inlineStr">
@@ -3800,7 +3687,6 @@
       <c r="F116" s="2" t="n">
         <v>125</v>
       </c>
-      <c r="G116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3813,7 +3699,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C117" s="1" t="n">
+      <c r="C117" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D117" t="inlineStr">
@@ -3829,7 +3715,6 @@
       <c r="F117" s="2" t="n">
         <v>555</v>
       </c>
-      <c r="G117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3842,7 +3727,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C118" s="1" t="n">
+      <c r="C118" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D118" t="inlineStr">
@@ -3858,7 +3743,6 @@
       <c r="F118" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="G118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3871,7 +3755,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C119" s="1" t="n">
+      <c r="C119" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D119" t="inlineStr">
@@ -3887,7 +3771,6 @@
       <c r="F119" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="G119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3900,7 +3783,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C120" s="1" t="n">
+      <c r="C120" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D120" t="inlineStr">
@@ -3916,7 +3799,6 @@
       <c r="F120" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="G120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3929,7 +3811,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C121" s="1" t="n">
+      <c r="C121" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D121" t="inlineStr">
@@ -3945,7 +3827,6 @@
       <c r="F121" s="2" t="n">
         <v>13.5</v>
       </c>
-      <c r="G121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3958,7 +3839,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C122" s="1" t="n">
+      <c r="C122" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D122" t="inlineStr">
@@ -3974,7 +3855,6 @@
       <c r="F122" s="2" t="n">
         <v>29.5</v>
       </c>
-      <c r="G122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3987,7 +3867,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C123" s="1" t="n">
+      <c r="C123" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D123" t="inlineStr">
@@ -4003,7 +3883,6 @@
       <c r="F123" s="2" t="n">
         <v>28.5</v>
       </c>
-      <c r="G123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4016,7 +3895,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C124" s="1" t="n">
+      <c r="C124" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D124" t="inlineStr">
@@ -4032,7 +3911,6 @@
       <c r="F124" s="2" t="n">
         <v>105</v>
       </c>
-      <c r="G124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4045,7 +3923,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C125" s="1" t="n">
+      <c r="C125" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D125" t="inlineStr">
@@ -4061,7 +3939,6 @@
       <c r="F125" s="2" t="n">
         <v>240</v>
       </c>
-      <c r="G125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4074,7 +3951,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C126" s="1" t="n">
+      <c r="C126" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D126" t="inlineStr">
@@ -4090,7 +3967,6 @@
       <c r="F126" s="2" t="n">
         <v>850</v>
       </c>
-      <c r="G126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4103,7 +3979,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C127" s="1" t="n">
+      <c r="C127" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D127" t="inlineStr">
@@ -4119,7 +3995,6 @@
       <c r="F127" s="2" t="n">
         <v>2300</v>
       </c>
-      <c r="G127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4132,7 +4007,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C128" s="1" t="n">
+      <c r="C128" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D128" t="inlineStr">
@@ -4148,7 +4023,6 @@
       <c r="F128" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4161,7 +4035,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C129" s="1" t="n">
+      <c r="C129" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D129" t="inlineStr">
@@ -4177,7 +4051,6 @@
       <c r="F129" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4190,7 +4063,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C130" s="1" t="n">
+      <c r="C130" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D130" t="inlineStr">
@@ -4206,7 +4079,6 @@
       <c r="F130" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="G130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4219,7 +4091,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C131" s="1" t="n">
+      <c r="C131" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D131" t="inlineStr">
@@ -4235,7 +4107,6 @@
       <c r="F131" s="2" t="n">
         <v>225</v>
       </c>
-      <c r="G131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4248,7 +4119,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C132" s="1" t="n">
+      <c r="C132" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D132" t="inlineStr">
@@ -4264,7 +4135,6 @@
       <c r="F132" s="2" t="n">
         <v>225</v>
       </c>
-      <c r="G132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4277,7 +4147,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C133" s="1" t="n">
+      <c r="C133" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D133" t="inlineStr">
@@ -4293,7 +4163,6 @@
       <c r="F133" s="2" t="n">
         <v>420</v>
       </c>
-      <c r="G133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4306,7 +4175,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C134" s="1" t="n">
+      <c r="C134" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D134" t="inlineStr">
@@ -4322,7 +4191,6 @@
       <c r="F134" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="G134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4335,7 +4203,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C135" s="1" t="n">
+      <c r="C135" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D135" t="inlineStr">
@@ -4351,7 +4219,6 @@
       <c r="F135" s="2" t="n">
         <v>125</v>
       </c>
-      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4364,7 +4231,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C136" s="1" t="n">
+      <c r="C136" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D136" t="inlineStr">
@@ -4380,7 +4247,6 @@
       <c r="F136" s="2" t="n">
         <v>555</v>
       </c>
-      <c r="G136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4393,7 +4259,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C137" s="1" t="n">
+      <c r="C137" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D137" t="inlineStr">
@@ -4409,7 +4275,6 @@
       <c r="F137" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="G137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4422,7 +4287,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C138" s="1" t="n">
+      <c r="C138" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D138" t="inlineStr">
@@ -4438,7 +4303,6 @@
       <c r="F138" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="G138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4451,7 +4315,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C139" s="1" t="n">
+      <c r="C139" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D139" t="inlineStr">
@@ -4467,7 +4331,6 @@
       <c r="F139" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="G139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4480,7 +4343,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C140" s="1" t="n">
+      <c r="C140" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D140" t="inlineStr">
@@ -4496,7 +4359,6 @@
       <c r="F140" s="2" t="n">
         <v>13.5</v>
       </c>
-      <c r="G140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4509,7 +4371,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C141" s="1" t="n">
+      <c r="C141" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D141" t="inlineStr">
@@ -4525,7 +4387,6 @@
       <c r="F141" s="2" t="n">
         <v>29.5</v>
       </c>
-      <c r="G141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4538,7 +4399,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C142" s="1" t="n">
+      <c r="C142" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D142" t="inlineStr">
@@ -4554,7 +4415,6 @@
       <c r="F142" s="2" t="n">
         <v>28.5</v>
       </c>
-      <c r="G142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4567,7 +4427,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C143" s="1" t="n">
+      <c r="C143" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D143" t="inlineStr">
@@ -4583,7 +4443,6 @@
       <c r="F143" s="2" t="n">
         <v>105</v>
       </c>
-      <c r="G143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4596,7 +4455,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C144" s="1" t="n">
+      <c r="C144" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D144" t="inlineStr">
@@ -4612,7 +4471,6 @@
       <c r="F144" s="2" t="n">
         <v>240</v>
       </c>
-      <c r="G144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4625,7 +4483,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C145" s="1" t="n">
+      <c r="C145" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D145" t="inlineStr">
@@ -4641,7 +4499,6 @@
       <c r="F145" s="2" t="n">
         <v>850</v>
       </c>
-      <c r="G145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -4654,7 +4511,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C146" s="1" t="n">
+      <c r="C146" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D146" t="inlineStr">
@@ -4670,7 +4527,6 @@
       <c r="F146" s="2" t="n">
         <v>2300</v>
       </c>
-      <c r="G146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4683,7 +4539,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C147" s="1" t="n">
+      <c r="C147" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D147" t="inlineStr">
@@ -4699,7 +4555,6 @@
       <c r="F147" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -4712,7 +4567,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C148" s="1" t="n">
+      <c r="C148" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D148" t="inlineStr">
@@ -4728,7 +4583,6 @@
       <c r="F148" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -4741,7 +4595,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C149" s="1" t="n">
+      <c r="C149" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D149" t="inlineStr">
@@ -4757,7 +4611,6 @@
       <c r="F149" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="G149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -4770,7 +4623,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C150" s="1" t="n">
+      <c r="C150" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D150" t="inlineStr">
@@ -4786,7 +4639,6 @@
       <c r="F150" s="2" t="n">
         <v>225</v>
       </c>
-      <c r="G150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -4799,7 +4651,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C151" s="1" t="n">
+      <c r="C151" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D151" t="inlineStr">
@@ -4815,7 +4667,6 @@
       <c r="F151" s="2" t="n">
         <v>225</v>
       </c>
-      <c r="G151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -4828,7 +4679,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C152" s="1" t="n">
+      <c r="C152" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D152" t="inlineStr">
@@ -4844,7 +4695,6 @@
       <c r="F152" s="2" t="n">
         <v>420</v>
       </c>
-      <c r="G152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -4857,7 +4707,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C153" s="1" t="n">
+      <c r="C153" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D153" t="inlineStr">
@@ -4873,7 +4723,6 @@
       <c r="F153" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="G153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -4886,7 +4735,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C154" s="1" t="n">
+      <c r="C154" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D154" t="inlineStr">
@@ -4902,7 +4751,6 @@
       <c r="F154" s="2" t="n">
         <v>125</v>
       </c>
-      <c r="G154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -4915,7 +4763,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C155" s="1" t="n">
+      <c r="C155" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D155" t="inlineStr">
@@ -4931,7 +4779,6 @@
       <c r="F155" s="2" t="n">
         <v>555</v>
       </c>
-      <c r="G155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -4944,7 +4791,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C156" s="1" t="n">
+      <c r="C156" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D156" t="inlineStr">
@@ -4960,7 +4807,6 @@
       <c r="F156" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="G156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -4973,7 +4819,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C157" s="1" t="n">
+      <c r="C157" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D157" t="inlineStr">
@@ -4989,7 +4835,6 @@
       <c r="F157" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="G157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -5002,7 +4847,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C158" s="1" t="n">
+      <c r="C158" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D158" t="inlineStr">
@@ -5018,7 +4863,6 @@
       <c r="F158" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="G158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5031,7 +4875,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C159" s="1" t="n">
+      <c r="C159" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D159" t="inlineStr">
@@ -5047,7 +4891,6 @@
       <c r="F159" s="2" t="n">
         <v>13.5</v>
       </c>
-      <c r="G159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -5060,7 +4903,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C160" s="1" t="n">
+      <c r="C160" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D160" t="inlineStr">
@@ -5076,7 +4919,6 @@
       <c r="F160" s="2" t="n">
         <v>29.5</v>
       </c>
-      <c r="G160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -5089,7 +4931,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C161" s="1" t="n">
+      <c r="C161" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D161" t="inlineStr">
@@ -5105,7 +4947,6 @@
       <c r="F161" s="2" t="n">
         <v>28.5</v>
       </c>
-      <c r="G161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -5118,7 +4959,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C162" s="1" t="n">
+      <c r="C162" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D162" t="inlineStr">
@@ -5134,7 +4975,6 @@
       <c r="F162" s="2" t="n">
         <v>105</v>
       </c>
-      <c r="G162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -5147,7 +4987,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C163" s="1" t="n">
+      <c r="C163" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D163" t="inlineStr">
@@ -5163,7 +5003,6 @@
       <c r="F163" s="2" t="n">
         <v>240</v>
       </c>
-      <c r="G163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -5176,7 +5015,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C164" s="1" t="n">
+      <c r="C164" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D164" t="inlineStr">
@@ -5192,7 +5031,6 @@
       <c r="F164" s="2" t="n">
         <v>850</v>
       </c>
-      <c r="G164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -5205,7 +5043,7 @@
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="C165" s="1" t="n">
+      <c r="C165" s="3" t="n">
         <v>45999</v>
       </c>
       <c r="D165" t="inlineStr">
@@ -5221,7 +5059,6 @@
       <c r="F165" s="2" t="n">
         <v>2300</v>
       </c>
-      <c r="G165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -5234,7 +5071,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C166" s="1" t="n">
+      <c r="C166" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D166" t="inlineStr">
@@ -5250,7 +5087,6 @@
       <c r="F166" s="2" t="n">
         <v>3534</v>
       </c>
-      <c r="G166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -5263,7 +5099,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C167" s="1" t="n">
+      <c r="C167" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D167" t="inlineStr">
@@ -5279,7 +5115,6 @@
       <c r="F167" s="2" t="n">
         <v>3534</v>
       </c>
-      <c r="G167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -5292,7 +5127,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C168" s="1" t="n">
+      <c r="C168" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D168" t="inlineStr">
@@ -5308,7 +5143,6 @@
       <c r="F168" s="2" t="n">
         <v>3534</v>
       </c>
-      <c r="G168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -5321,7 +5155,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C169" s="1" t="n">
+      <c r="C169" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D169" t="inlineStr">
@@ -5337,7 +5171,6 @@
       <c r="F169" s="2" t="n">
         <v>2584</v>
       </c>
-      <c r="G169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -5350,7 +5183,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C170" s="1" t="n">
+      <c r="C170" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D170" t="inlineStr">
@@ -5366,7 +5199,6 @@
       <c r="F170" s="2" t="n">
         <v>725</v>
       </c>
-      <c r="G170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -5379,7 +5211,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C171" s="1" t="n">
+      <c r="C171" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D171" t="inlineStr">
@@ -5395,7 +5227,6 @@
       <c r="F171" s="2" t="n">
         <v>725</v>
       </c>
-      <c r="G171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -5408,7 +5239,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C172" s="1" t="n">
+      <c r="C172" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D172" t="inlineStr">
@@ -5424,7 +5255,6 @@
       <c r="F172" s="2" t="n">
         <v>725</v>
       </c>
-      <c r="G172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -5437,7 +5267,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C173" s="1" t="n">
+      <c r="C173" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D173" t="inlineStr">
@@ -5453,7 +5283,6 @@
       <c r="F173" s="2" t="n">
         <v>725</v>
       </c>
-      <c r="G173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -5466,7 +5295,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C174" s="1" t="n">
+      <c r="C174" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D174" t="inlineStr">
@@ -5482,7 +5311,6 @@
       <c r="F174" s="2" t="n">
         <v>2703</v>
       </c>
-      <c r="G174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -5495,7 +5323,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C175" s="1" t="n">
+      <c r="C175" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D175" t="inlineStr">
@@ -5511,7 +5339,6 @@
       <c r="F175" s="2" t="n">
         <v>1025</v>
       </c>
-      <c r="G175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -5524,7 +5351,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C176" s="1" t="n">
+      <c r="C176" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D176" t="inlineStr">
@@ -5540,7 +5367,6 @@
       <c r="F176" s="2" t="n">
         <v>1025</v>
       </c>
-      <c r="G176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -5553,7 +5379,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C177" s="1" t="n">
+      <c r="C177" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D177" t="inlineStr">
@@ -5569,7 +5395,6 @@
       <c r="F177" s="2" t="n">
         <v>1025</v>
       </c>
-      <c r="G177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -5582,7 +5407,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C178" s="1" t="n">
+      <c r="C178" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D178" t="inlineStr">
@@ -5598,7 +5423,6 @@
       <c r="F178" s="2" t="n">
         <v>1025</v>
       </c>
-      <c r="G178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -5611,7 +5435,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C179" s="1" t="n">
+      <c r="C179" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D179" t="inlineStr">
@@ -5627,7 +5451,6 @@
       <c r="F179" s="2" t="n">
         <v>2470</v>
       </c>
-      <c r="G179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -5640,7 +5463,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C180" s="1" t="n">
+      <c r="C180" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D180" t="inlineStr">
@@ -5656,7 +5479,6 @@
       <c r="F180" s="2" t="n">
         <v>825</v>
       </c>
-      <c r="G180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -5669,7 +5491,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C181" s="1" t="n">
+      <c r="C181" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D181" t="inlineStr">
@@ -5685,7 +5507,6 @@
       <c r="F181" s="2" t="n">
         <v>825</v>
       </c>
-      <c r="G181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -5698,7 +5519,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C182" s="1" t="n">
+      <c r="C182" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D182" t="inlineStr">
@@ -5714,7 +5535,6 @@
       <c r="F182" s="2" t="n">
         <v>825</v>
       </c>
-      <c r="G182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -5727,7 +5547,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C183" s="1" t="n">
+      <c r="C183" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="D183" t="inlineStr">
@@ -5743,7 +5563,6 @@
       <c r="F183" s="2" t="n">
         <v>825</v>
       </c>
-      <c r="G183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -5756,7 +5575,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C184" s="1" t="n">
+      <c r="C184" s="3" t="n">
         <v>45427</v>
       </c>
       <c r="D184" t="inlineStr">
@@ -5772,7 +5591,6 @@
       <c r="F184" s="2" t="n">
         <v>547</v>
       </c>
-      <c r="G184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -5785,7 +5603,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C185" s="1" t="n">
+      <c r="C185" s="3" t="n">
         <v>45427</v>
       </c>
       <c r="D185" t="inlineStr">
@@ -5801,7 +5619,6 @@
       <c r="F185" s="2" t="n">
         <v>547</v>
       </c>
-      <c r="G185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -5814,7 +5631,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C186" s="1" t="n">
+      <c r="C186" s="3" t="n">
         <v>45427</v>
       </c>
       <c r="D186" t="inlineStr">
@@ -5830,7 +5647,6 @@
       <c r="F186" s="2" t="n">
         <v>547</v>
       </c>
-      <c r="G186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -5843,7 +5659,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C187" s="1" t="n">
+      <c r="C187" s="3" t="n">
         <v>45427</v>
       </c>
       <c r="D187" t="inlineStr">
@@ -5859,7 +5675,6 @@
       <c r="F187" s="2" t="n">
         <v>547</v>
       </c>
-      <c r="G187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -5872,7 +5687,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C188" s="1" t="n">
+      <c r="C188" s="3" t="n">
         <v>45792</v>
       </c>
       <c r="D188" t="inlineStr">
@@ -5888,7 +5703,6 @@
       <c r="F188" s="2" t="n">
         <v>3210</v>
       </c>
-      <c r="G188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -5901,7 +5715,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C189" s="1" t="n">
+      <c r="C189" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D189" t="inlineStr">
@@ -5917,7 +5731,6 @@
       <c r="F189" s="2" t="n">
         <v>8567</v>
       </c>
-      <c r="G189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -5930,7 +5743,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C190" s="1" t="n">
+      <c r="C190" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D190" t="inlineStr">
@@ -5946,7 +5759,6 @@
       <c r="F190" s="2" t="n">
         <v>501</v>
       </c>
-      <c r="G190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -5959,7 +5771,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C191" s="1" t="n">
+      <c r="C191" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D191" t="inlineStr">
@@ -5975,7 +5787,6 @@
       <c r="F191" s="2" t="n">
         <v>8926</v>
       </c>
-      <c r="G191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -5988,7 +5799,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C192" s="1" t="n">
+      <c r="C192" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D192" t="inlineStr">
@@ -6004,7 +5815,6 @@
       <c r="F192" s="2" t="n">
         <v>735</v>
       </c>
-      <c r="G192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -6017,7 +5827,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C193" s="1" t="n">
+      <c r="C193" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D193" t="inlineStr">
@@ -6033,7 +5843,6 @@
       <c r="F193" s="2" t="n">
         <v>9330</v>
       </c>
-      <c r="G193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -6046,7 +5855,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C194" s="1" t="n">
+      <c r="C194" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D194" t="inlineStr">
@@ -6062,7 +5871,6 @@
       <c r="F194" s="2" t="n">
         <v>526</v>
       </c>
-      <c r="G194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -6075,7 +5883,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C195" s="1" t="n">
+      <c r="C195" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D195" t="inlineStr">
@@ -6091,7 +5899,6 @@
       <c r="F195" s="2" t="n">
         <v>430</v>
       </c>
-      <c r="G195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -6104,7 +5911,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C196" s="1" t="n">
+      <c r="C196" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="D196" t="inlineStr">
@@ -6120,7 +5927,6 @@
       <c r="F196" s="2" t="n">
         <v>300</v>
       </c>
-      <c r="G196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -6133,7 +5939,7 @@
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C197" s="1" t="n">
+      <c r="C197" s="3" t="n">
         <v>46153</v>
       </c>
       <c r="D197" t="inlineStr">
@@ -6166,7 +5972,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C198" s="1" t="n">
+      <c r="C198" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D198" t="inlineStr">
@@ -6182,7 +5988,6 @@
       <c r="F198" s="2" t="n">
         <v>11550</v>
       </c>
-      <c r="G198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -6195,7 +6000,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C199" s="1" t="n">
+      <c r="C199" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D199" t="inlineStr">
@@ -6211,7 +6016,6 @@
       <c r="F199" s="2" t="n">
         <v>439</v>
       </c>
-      <c r="G199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -6224,7 +6028,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C200" s="1" t="n">
+      <c r="C200" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D200" t="inlineStr">
@@ -6240,7 +6044,6 @@
       <c r="F200" s="2" t="n">
         <v>439</v>
       </c>
-      <c r="G200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -6253,7 +6056,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C201" s="1" t="n">
+      <c r="C201" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D201" t="inlineStr">
@@ -6269,7 +6072,6 @@
       <c r="F201" s="2" t="n">
         <v>437</v>
       </c>
-      <c r="G201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -6282,7 +6084,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C202" s="1" t="n">
+      <c r="C202" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D202" t="inlineStr">
@@ -6298,7 +6100,6 @@
       <c r="F202" s="2" t="n">
         <v>428</v>
       </c>
-      <c r="G202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -6311,7 +6112,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C203" s="1" t="n">
+      <c r="C203" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D203" t="inlineStr">
@@ -6327,7 +6128,6 @@
       <c r="F203" s="2" t="n">
         <v>663</v>
       </c>
-      <c r="G203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -6340,7 +6140,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C204" s="1" t="n">
+      <c r="C204" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D204" t="inlineStr">
@@ -6356,7 +6156,6 @@
       <c r="F204" s="2" t="n">
         <v>11684</v>
       </c>
-      <c r="G204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -6369,7 +6168,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C205" s="1" t="n">
+      <c r="C205" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D205" t="inlineStr">
@@ -6385,7 +6184,6 @@
       <c r="F205" s="2" t="n">
         <v>374</v>
       </c>
-      <c r="G205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -6398,7 +6196,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C206" s="1" t="n">
+      <c r="C206" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D206" t="inlineStr">
@@ -6414,7 +6212,6 @@
       <c r="F206" s="2" t="n">
         <v>1277</v>
       </c>
-      <c r="G206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -6427,7 +6224,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C207" s="1" t="n">
+      <c r="C207" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D207" t="inlineStr">
@@ -6443,7 +6240,6 @@
       <c r="F207" s="2" t="n">
         <v>1277</v>
       </c>
-      <c r="G207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -6456,7 +6252,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C208" s="1" t="n">
+      <c r="C208" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D208" t="inlineStr">
@@ -6472,7 +6268,6 @@
       <c r="F208" s="2" t="n">
         <v>12346</v>
       </c>
-      <c r="G208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -6485,7 +6280,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C209" s="1" t="n">
+      <c r="C209" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D209" t="inlineStr">
@@ -6501,7 +6296,6 @@
       <c r="F209" s="2" t="n">
         <v>692</v>
       </c>
-      <c r="G209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -6514,7 +6308,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C210" s="1" t="n">
+      <c r="C210" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D210" t="inlineStr">
@@ -6530,7 +6324,6 @@
       <c r="F210" s="2" t="n">
         <v>714</v>
       </c>
-      <c r="G210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -6543,7 +6336,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C211" s="1" t="n">
+      <c r="C211" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D211" t="inlineStr">
@@ -6559,7 +6352,6 @@
       <c r="F211" s="2" t="n">
         <v>714</v>
       </c>
-      <c r="G211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -6572,7 +6364,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C212" s="1" t="n">
+      <c r="C212" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D212" t="inlineStr">
@@ -6588,7 +6380,6 @@
       <c r="F212" s="2" t="n">
         <v>570</v>
       </c>
-      <c r="G212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -6601,7 +6392,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C213" s="1" t="n">
+      <c r="C213" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D213" t="inlineStr">
@@ -6617,7 +6408,6 @@
       <c r="F213" s="2" t="n">
         <v>12646</v>
       </c>
-      <c r="G213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -6630,7 +6420,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C214" s="1" t="n">
+      <c r="C214" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D214" t="inlineStr">
@@ -6646,7 +6436,6 @@
       <c r="F214" s="2" t="n">
         <v>720</v>
       </c>
-      <c r="G214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -6659,7 +6448,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C215" s="1" t="n">
+      <c r="C215" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D215" t="inlineStr">
@@ -6675,7 +6464,6 @@
       <c r="F215" s="2" t="n">
         <v>720</v>
       </c>
-      <c r="G215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -6688,7 +6476,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C216" s="1" t="n">
+      <c r="C216" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D216" t="inlineStr">
@@ -6704,7 +6492,6 @@
       <c r="F216" s="2" t="n">
         <v>720</v>
       </c>
-      <c r="G216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -6717,7 +6504,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C217" s="1" t="n">
+      <c r="C217" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D217" t="inlineStr">
@@ -6733,7 +6520,6 @@
       <c r="F217" s="2" t="n">
         <v>4368</v>
       </c>
-      <c r="G217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -6746,7 +6532,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C218" s="1" t="n">
+      <c r="C218" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D218" t="inlineStr">
@@ -6762,7 +6548,6 @@
       <c r="F218" s="2" t="n">
         <v>4368</v>
       </c>
-      <c r="G218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -6775,7 +6560,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C219" s="1" t="n">
+      <c r="C219" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D219" t="inlineStr">
@@ -6791,7 +6576,6 @@
       <c r="F219" s="2" t="n">
         <v>4368</v>
       </c>
-      <c r="G219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -6804,7 +6588,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C220" s="1" t="n">
+      <c r="C220" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D220" t="inlineStr">
@@ -6820,7 +6604,6 @@
       <c r="F220" s="2" t="n">
         <v>14023</v>
       </c>
-      <c r="G220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -6833,7 +6616,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C221" s="1" t="n">
+      <c r="C221" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D221" t="inlineStr">
@@ -6849,7 +6632,6 @@
       <c r="F221" s="2" t="n">
         <v>559</v>
       </c>
-      <c r="G221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -6862,7 +6644,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C222" s="1" t="n">
+      <c r="C222" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D222" t="inlineStr">
@@ -6878,7 +6660,6 @@
       <c r="F222" s="2" t="n">
         <v>619</v>
       </c>
-      <c r="G222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -6891,7 +6672,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C223" s="1" t="n">
+      <c r="C223" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D223" t="inlineStr">
@@ -6907,7 +6688,6 @@
       <c r="F223" s="2" t="n">
         <v>657</v>
       </c>
-      <c r="G223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -6920,7 +6700,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C224" s="1" t="n">
+      <c r="C224" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D224" t="inlineStr">
@@ -6936,7 +6716,6 @@
       <c r="F224" s="2" t="n">
         <v>14913</v>
       </c>
-      <c r="G224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -6949,7 +6728,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C225" s="1" t="n">
+      <c r="C225" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D225" t="inlineStr">
@@ -6965,7 +6744,6 @@
       <c r="F225" s="2" t="n">
         <v>720</v>
       </c>
-      <c r="G225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -6978,7 +6756,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C226" s="1" t="n">
+      <c r="C226" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D226" t="inlineStr">
@@ -6994,7 +6772,6 @@
       <c r="F226" s="2" t="n">
         <v>720</v>
       </c>
-      <c r="G226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -7007,7 +6784,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C227" s="1" t="n">
+      <c r="C227" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="D227" t="inlineStr">
@@ -7023,7 +6800,6 @@
       <c r="F227" s="2" t="n">
         <v>720</v>
       </c>
-      <c r="G227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -7036,7 +6812,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C228" s="1" t="n">
+      <c r="C228" s="3" t="n">
         <v>45839</v>
       </c>
       <c r="D228" t="inlineStr">
@@ -7052,7 +6828,6 @@
       <c r="F228" s="2" t="n">
         <v>5273</v>
       </c>
-      <c r="G228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -7065,7 +6840,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C229" s="1" t="n">
+      <c r="C229" s="3" t="n">
         <v>45839</v>
       </c>
       <c r="D229" t="inlineStr">
@@ -7081,7 +6856,6 @@
       <c r="F229" s="2" t="n">
         <v>5659</v>
       </c>
-      <c r="G229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -7094,7 +6868,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C230" s="1" t="n">
+      <c r="C230" s="3" t="n">
         <v>45839</v>
       </c>
       <c r="D230" t="inlineStr">
@@ -7110,7 +6884,6 @@
       <c r="F230" s="2" t="n">
         <v>5955</v>
       </c>
-      <c r="G230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -7123,7 +6896,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C231" s="1" t="n">
+      <c r="C231" s="3" t="n">
         <v>45992</v>
       </c>
       <c r="D231" t="inlineStr">
@@ -7139,7 +6912,6 @@
       <c r="F231" s="2" t="n">
         <v>4925</v>
       </c>
-      <c r="G231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -7152,7 +6924,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C232" s="1" t="n">
+      <c r="C232" s="3" t="n">
         <v>45992</v>
       </c>
       <c r="D232" t="inlineStr">
@@ -7168,7 +6940,6 @@
       <c r="F232" s="2" t="n">
         <v>5286</v>
       </c>
-      <c r="G232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -7181,7 +6952,7 @@
           <t>Foundation</t>
         </is>
       </c>
-      <c r="C233" s="1" t="n">
+      <c r="C233" s="3" t="n">
         <v>45992</v>
       </c>
       <c r="D233" t="inlineStr">
@@ -7197,7 +6968,105 @@
       <c r="F233" s="2" t="n">
         <v>5562</v>
       </c>
-      <c r="G233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Edgeview Estates</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Plan Pricing</t>
+        </is>
+      </c>
+      <c r="C234" s="3" t="n">
+        <v>46327</v>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Vista</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F234" s="2" t="n">
+        <v>3306</v>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Edgeview Estates</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Plan Pricing</t>
+        </is>
+      </c>
+      <c r="C235" s="3" t="n">
+        <v>46327</v>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Horizon</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F235" s="2" t="n">
+        <v>3577</v>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Edgeview Estates</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Plan Pricing</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="n">
+        <v>46327</v>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Summit</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F236" s="2" t="n">
+        <v>3140</v>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Skyeview Mesa unit pricing per Century pricing schedule 5002079 eff 10/13/2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D6wjrb1spFgY1HgqZrWwPC
</commit_message>
<xml_diff>
--- a/CenturyCommunitiesContracts1.xlsx
+++ b/CenturyCommunitiesContracts1.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -4064,7 +4063,7 @@
         </is>
       </c>
       <c r="C130" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -4077,7 +4076,7 @@
         </is>
       </c>
       <c r="F130" s="2" t="n">
-        <v>375</v>
+        <v>365.63</v>
       </c>
     </row>
     <row r="131">
@@ -4148,7 +4147,7 @@
         </is>
       </c>
       <c r="C133" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
@@ -4161,7 +4160,7 @@
         </is>
       </c>
       <c r="F133" s="2" t="n">
-        <v>420</v>
+        <v>409.5</v>
       </c>
     </row>
     <row r="134">
@@ -4176,7 +4175,7 @@
         </is>
       </c>
       <c r="C134" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -4189,7 +4188,7 @@
         </is>
       </c>
       <c r="F134" s="2" t="n">
-        <v>450</v>
+        <v>438.75</v>
       </c>
     </row>
     <row r="135">
@@ -4204,7 +4203,7 @@
         </is>
       </c>
       <c r="C135" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -4217,7 +4216,7 @@
         </is>
       </c>
       <c r="F135" s="2" t="n">
-        <v>125</v>
+        <v>121.88</v>
       </c>
     </row>
     <row r="136">
@@ -4232,7 +4231,7 @@
         </is>
       </c>
       <c r="C136" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -4245,7 +4244,7 @@
         </is>
       </c>
       <c r="F136" s="2" t="n">
-        <v>555</v>
+        <v>541.13</v>
       </c>
     </row>
     <row r="137">
@@ -4288,7 +4287,7 @@
         </is>
       </c>
       <c r="C138" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -4301,7 +4300,7 @@
         </is>
       </c>
       <c r="F138" s="2" t="n">
-        <v>90</v>
+        <v>87.75</v>
       </c>
     </row>
     <row r="139">
@@ -4316,7 +4315,7 @@
         </is>
       </c>
       <c r="C139" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
@@ -4329,7 +4328,7 @@
         </is>
       </c>
       <c r="F139" s="2" t="n">
-        <v>81</v>
+        <v>78.98</v>
       </c>
     </row>
     <row r="140">
@@ -4400,7 +4399,7 @@
         </is>
       </c>
       <c r="C142" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -4413,7 +4412,7 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>28.5</v>
+        <v>27.79</v>
       </c>
     </row>
     <row r="143">
@@ -4456,7 +4455,7 @@
         </is>
       </c>
       <c r="C144" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
@@ -4469,7 +4468,7 @@
         </is>
       </c>
       <c r="F144" s="2" t="n">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="145">

</xml_diff>

<commit_message>
Century: Skyeview Terra landscape pricing 5002080 (eff 10/13/2026) and Skyeview Arroyo concrete 5002082 (eff 10/1/2026)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D6wjrb1spFgY1HgqZrWwPC
</commit_message>
<xml_diff>
--- a/CenturyCommunitiesContracts1.xlsx
+++ b/CenturyCommunitiesContracts1.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G236"/>
+  <dimension ref="A1:G239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4595,7 +4595,7 @@
         </is>
       </c>
       <c r="C149" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -4608,7 +4608,7 @@
         </is>
       </c>
       <c r="F149" s="2" t="n">
-        <v>375</v>
+        <v>365.63</v>
       </c>
     </row>
     <row r="150">
@@ -4679,7 +4679,7 @@
         </is>
       </c>
       <c r="C152" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -4692,7 +4692,7 @@
         </is>
       </c>
       <c r="F152" s="2" t="n">
-        <v>420</v>
+        <v>409.5</v>
       </c>
     </row>
     <row r="153">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="C153" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -4720,7 +4720,7 @@
         </is>
       </c>
       <c r="F153" s="2" t="n">
-        <v>450</v>
+        <v>438.75</v>
       </c>
     </row>
     <row r="154">
@@ -4735,7 +4735,7 @@
         </is>
       </c>
       <c r="C154" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
         </is>
       </c>
       <c r="F154" s="2" t="n">
-        <v>125</v>
+        <v>121.88</v>
       </c>
     </row>
     <row r="155">
@@ -4763,7 +4763,7 @@
         </is>
       </c>
       <c r="C155" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -4776,7 +4776,7 @@
         </is>
       </c>
       <c r="F155" s="2" t="n">
-        <v>555</v>
+        <v>541.13</v>
       </c>
     </row>
     <row r="156">
@@ -4819,7 +4819,7 @@
         </is>
       </c>
       <c r="C157" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
@@ -4832,7 +4832,7 @@
         </is>
       </c>
       <c r="F157" s="2" t="n">
-        <v>90</v>
+        <v>87.75</v>
       </c>
     </row>
     <row r="158">
@@ -4847,7 +4847,7 @@
         </is>
       </c>
       <c r="C158" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D158" t="inlineStr">
         <is>
@@ -4860,7 +4860,7 @@
         </is>
       </c>
       <c r="F158" s="2" t="n">
-        <v>81</v>
+        <v>78.98</v>
       </c>
     </row>
     <row r="159">
@@ -4931,7 +4931,7 @@
         </is>
       </c>
       <c r="C161" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D161" t="inlineStr">
         <is>
@@ -4944,7 +4944,7 @@
         </is>
       </c>
       <c r="F161" s="2" t="n">
-        <v>28.5</v>
+        <v>27.79</v>
       </c>
     </row>
     <row r="162">
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="C163" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -5000,7 +5000,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="164">
@@ -6971,97 +6971,181 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Edgeview Estates</t>
+          <t>Skyeview - Arroyo - Concrete</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="C234" s="3" t="n">
-        <v>46327</v>
+        <v>46296</v>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>Vista</t>
+          <t>Beverly</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F234" s="2" t="n">
-        <v>3306</v>
-      </c>
-      <c r="G234" t="inlineStr">
-        <is>
-          <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
-        </is>
+        <v>4802</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Edgeview Estates</t>
+          <t>Skyeview - Arroyo - Concrete</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="C235" s="3" t="n">
-        <v>46327</v>
+        <v>46296</v>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>Horizon</t>
+          <t>Captiva</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F235" s="2" t="n">
-        <v>3577</v>
-      </c>
-      <c r="G235" t="inlineStr">
-        <is>
-          <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
-        </is>
+        <v>5154</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Delray</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F236" s="2" t="n">
+        <v>5423</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
           <t>Edgeview Estates</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr">
+      <c r="B237" t="inlineStr">
         <is>
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C236" s="3" t="n">
+      <c r="C237" s="3" t="n">
         <v>46327</v>
       </c>
-      <c r="D236" t="inlineStr">
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Vista</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F237" s="2" t="n">
+        <v>3306</v>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Edgeview Estates</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Plan Pricing</t>
+        </is>
+      </c>
+      <c r="C238" s="3" t="n">
+        <v>46327</v>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Horizon</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="n">
+        <v>3577</v>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Edgeview Estates</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Plan Pricing</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="n">
+        <v>46327</v>
+      </c>
+      <c r="D239" t="inlineStr">
         <is>
           <t>Summit</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr">
+      <c r="E239" t="inlineStr">
         <is>
           <t>Pavers</t>
         </is>
       </c>
-      <c r="F236" s="2" t="n">
+      <c r="F239" s="2" t="n">
         <v>3140</v>
       </c>
-      <c r="G236" t="inlineStr">
+      <c r="G239" t="inlineStr">
         <is>
           <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
         </is>

</xml_diff>

<commit_message>
Century Mesa/Terra unit pricing: keep full 19-item list on both the 12/8/2025 and 10/13/2026 dates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D6wjrb1spFgY1HgqZrWwPC
</commit_message>
<xml_diff>
--- a/CenturyCommunitiesContracts1.xlsx
+++ b/CenturyCommunitiesContracts1.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G239"/>
+  <dimension ref="A1:G277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4063,7 +4063,7 @@
         </is>
       </c>
       <c r="C130" s="3" t="n">
-        <v>46308</v>
+        <v>45999</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -4076,7 +4076,7 @@
         </is>
       </c>
       <c r="F130" s="2" t="n">
-        <v>365.63</v>
+        <v>375</v>
       </c>
     </row>
     <row r="131">
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="C133" s="3" t="n">
-        <v>46308</v>
+        <v>45999</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="F133" s="2" t="n">
-        <v>409.5</v>
+        <v>420</v>
       </c>
     </row>
     <row r="134">
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="C134" s="3" t="n">
-        <v>46308</v>
+        <v>45999</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -4188,7 +4188,7 @@
         </is>
       </c>
       <c r="F134" s="2" t="n">
-        <v>438.75</v>
+        <v>450</v>
       </c>
     </row>
     <row r="135">
@@ -4203,7 +4203,7 @@
         </is>
       </c>
       <c r="C135" s="3" t="n">
-        <v>46308</v>
+        <v>45999</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -4216,7 +4216,7 @@
         </is>
       </c>
       <c r="F135" s="2" t="n">
-        <v>121.88</v>
+        <v>125</v>
       </c>
     </row>
     <row r="136">
@@ -4231,7 +4231,7 @@
         </is>
       </c>
       <c r="C136" s="3" t="n">
-        <v>46308</v>
+        <v>45999</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -4244,7 +4244,7 @@
         </is>
       </c>
       <c r="F136" s="2" t="n">
-        <v>541.13</v>
+        <v>555</v>
       </c>
     </row>
     <row r="137">
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="C138" s="3" t="n">
-        <v>46308</v>
+        <v>45999</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -4300,7 +4300,7 @@
         </is>
       </c>
       <c r="F138" s="2" t="n">
-        <v>87.75</v>
+        <v>90</v>
       </c>
     </row>
     <row r="139">
@@ -4315,7 +4315,7 @@
         </is>
       </c>
       <c r="C139" s="3" t="n">
-        <v>46308</v>
+        <v>45999</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
@@ -4328,7 +4328,7 @@
         </is>
       </c>
       <c r="F139" s="2" t="n">
-        <v>78.98</v>
+        <v>81</v>
       </c>
     </row>
     <row r="140">
@@ -4399,7 +4399,7 @@
         </is>
       </c>
       <c r="C142" s="3" t="n">
-        <v>46308</v>
+        <v>45999</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>27.79</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="143">
@@ -4455,7 +4455,7 @@
         </is>
       </c>
       <c r="C144" s="3" t="n">
-        <v>46308</v>
+        <v>45999</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
@@ -4468,7 +4468,7 @@
         </is>
       </c>
       <c r="F144" s="2" t="n">
-        <v>234</v>
+        <v>240</v>
       </c>
     </row>
     <row r="145">
@@ -4530,7 +4530,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4539,7 +4539,7 @@
         </is>
       </c>
       <c r="C147" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -4558,7 +4558,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="C148" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -4586,7 +4586,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4614,7 +4614,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4623,7 +4623,7 @@
         </is>
       </c>
       <c r="C150" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
@@ -4642,7 +4642,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4651,7 +4651,7 @@
         </is>
       </c>
       <c r="C151" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -4670,7 +4670,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4698,7 +4698,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4726,7 +4726,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4754,7 +4754,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4782,7 +4782,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4791,7 +4791,7 @@
         </is>
       </c>
       <c r="C156" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
@@ -4810,7 +4810,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4838,7 +4838,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4866,7 +4866,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4875,7 +4875,7 @@
         </is>
       </c>
       <c r="C159" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -4894,7 +4894,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4903,7 +4903,7 @@
         </is>
       </c>
       <c r="C160" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
@@ -4922,7 +4922,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4950,7 +4950,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4959,7 +4959,7 @@
         </is>
       </c>
       <c r="C162" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
@@ -4978,7 +4978,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -5006,7 +5006,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -5015,7 +5015,7 @@
         </is>
       </c>
       <c r="C164" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
@@ -5034,7 +5034,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Skyeview - Terra</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -5043,7 +5043,7 @@
         </is>
       </c>
       <c r="C165" s="3" t="n">
-        <v>45999</v>
+        <v>46308</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
@@ -5062,1113 +5062,1108 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C166" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>1635</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>GF0000ATEX Final Grade Attached, End Unit (LS)</t>
         </is>
       </c>
       <c r="F166" s="2" t="n">
-        <v>3534</v>
+        <v>200</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C167" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>1742</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>GF0000ATIN Final Grade Attached, Interior Unit (LS)</t>
         </is>
       </c>
       <c r="F167" s="2" t="n">
-        <v>3534</v>
+        <v>200</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C168" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>1816</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>GF0000DTCH Final Grade Detached (LS)</t>
         </is>
       </c>
       <c r="F168" s="2" t="n">
-        <v>3534</v>
+        <v>375</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C169" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>1635</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>GR0000ATEX Rough Grade Attached, End Unit (LS)</t>
         </is>
       </c>
       <c r="F169" s="2" t="n">
-        <v>2584</v>
+        <v>225</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C170" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>1635</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>PVO-CP0206 Patio Cover</t>
+          <t>GR0000ATIN Rough Grade Attached, Interior Unit (LS)</t>
         </is>
       </c>
       <c r="F170" s="2" t="n">
-        <v>725</v>
+        <v>225</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C171" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>1635</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>PVO-AL0200 Alumawood Patio Cover - Lattice</t>
+          <t>GR0000DTCH Rough Grade Detached (LS)</t>
         </is>
       </c>
       <c r="F171" s="2" t="n">
-        <v>725</v>
+        <v>420</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C172" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>1635</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>PVO-AL0250 Alumawood Patio Cover - Solid</t>
+          <t>GR0000HAUL Rough Grade Haul Off (LS)</t>
         </is>
       </c>
       <c r="F172" s="2" t="n">
-        <v>725</v>
+        <v>450</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C173" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1635</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>PVO-CP155 Patio Pavers Only</t>
+          <t>LI0000TIMR Irrigation Timer (EA)</t>
         </is>
       </c>
       <c r="F173" s="2" t="n">
-        <v>725</v>
+        <v>125</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C174" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>1742</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>LI0000ZONE Irrigation Per Zone (EA)</t>
         </is>
       </c>
       <c r="F174" s="2" t="n">
-        <v>2703</v>
+        <v>555</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C175" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>1742</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>PVO-CP0206 Patio Cover</t>
+          <t>LLG000BLDR Ground Cover Boulder (EA)</t>
         </is>
       </c>
       <c r="F175" s="2" t="n">
-        <v>1025</v>
+        <v>69</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C176" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>1742</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>PVO-AL0200 Alumawood Patio Cover - Lattice</t>
+          <t>LLG000CR24 Ground Cover 2-4in Cobble Rock (CY)</t>
         </is>
       </c>
       <c r="F176" s="2" t="n">
-        <v>1025</v>
+        <v>90</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C177" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>1742</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>PVO-AL0250 Alumawood Patio Cover - Solid</t>
+          <t>LLG3QIROCK Ground Cover 3/4in Rock (CY)</t>
         </is>
       </c>
       <c r="F177" s="2" t="n">
-        <v>1025</v>
+        <v>81</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C178" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>1742</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>PVO-CP155 Patio Pavers Only</t>
+          <t>LLS01GSHRB Shrubs &amp; Plants 1-gallon (EA)</t>
         </is>
       </c>
       <c r="F178" s="2" t="n">
-        <v>1025</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C179" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>1816</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>LLS03GSHRB Shrubs &amp; Plants 3-gallon (EA)</t>
         </is>
       </c>
       <c r="F179" s="2" t="n">
-        <v>2470</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C180" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>1816</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>PVO-CP0206 Patio Cover</t>
+          <t>LLS05GSHRB Shrubs &amp; Plants 5-gallon (EA)</t>
         </is>
       </c>
       <c r="F180" s="2" t="n">
-        <v>825</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C181" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>1816</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>PVO-AL0200 Alumawood Patio Cover - Lattice</t>
+          <t>LLS15GSHRB Shrubs &amp; Plants 15-gallon (EA)</t>
         </is>
       </c>
       <c r="F181" s="2" t="n">
-        <v>825</v>
+        <v>105</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C182" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>1816</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>PVO-AL0250 Alumawood Patio Cover - Solid</t>
+          <t>LLT01ITREE Tree 1in Caliper (EA)</t>
         </is>
       </c>
       <c r="F182" s="2" t="n">
-        <v>825</v>
+        <v>240</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C183" s="3" t="n">
-        <v>45748</v>
+        <v>45999</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>1816</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>PVO-CP155 Patio Pavers Only</t>
+          <t>LLT02ITREE Tree 2in Caliper (EA)</t>
         </is>
       </c>
       <c r="F183" s="2" t="n">
-        <v>825</v>
+        <v>850</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Union Village</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C184" s="3" t="n">
-        <v>45427</v>
+        <v>45999</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>1405</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>LLT03ITREE Tree 3in Caliper (EA)</t>
         </is>
       </c>
       <c r="F184" s="2" t="n">
-        <v>547</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Union Village</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C185" s="3" t="n">
-        <v>45427</v>
+        <v>46308</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>1478</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>GF0000ATEX Final Grade Attached, End Unit (LS)</t>
         </is>
       </c>
       <c r="F185" s="2" t="n">
-        <v>547</v>
+        <v>200</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Union Village</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C186" s="3" t="n">
-        <v>45427</v>
+        <v>46308</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>1478E</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>GF0000ATIN Final Grade Attached, Interior Unit (LS)</t>
         </is>
       </c>
       <c r="F186" s="2" t="n">
-        <v>547</v>
+        <v>200</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Union Village</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C187" s="3" t="n">
-        <v>45427</v>
+        <v>46308</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>1479</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>GF0000DTCH Final Grade Detached (LS)</t>
         </is>
       </c>
       <c r="F187" s="2" t="n">
-        <v>547</v>
+        <v>365.63</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Ishani Ridge (Century Complete)</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C188" s="3" t="n">
-        <v>45792</v>
+        <v>46308</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>GR0000ATEX Rough Grade Attached, End Unit (LS)</t>
         </is>
       </c>
       <c r="F188" s="2" t="n">
-        <v>3210</v>
+        <v>225</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C189" s="3" t="n">
-        <v>46296</v>
+        <v>46308</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>1635</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>GR0000ATIN Rough Grade Attached, Interior Unit (LS)</t>
         </is>
       </c>
       <c r="F189" s="2" t="n">
-        <v>8567</v>
+        <v>225</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C190" s="3" t="n">
-        <v>46296</v>
+        <v>46308</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>1635</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>CP0206 - Patio Cover A - Elevation A</t>
+          <t>GR0000DTCH Rough Grade Detached (LS)</t>
         </is>
       </c>
       <c r="F190" s="2" t="n">
-        <v>501</v>
+        <v>409.5</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C191" s="3" t="n">
-        <v>46296</v>
+        <v>46308</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>1742</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>GR0000HAUL Rough Grade Haul Off (LS)</t>
         </is>
       </c>
       <c r="F191" s="2" t="n">
-        <v>8926</v>
+        <v>438.75</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C192" s="3" t="n">
-        <v>46296</v>
+        <v>46308</v>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>1742</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>CP0206 - Patio Cover A - Elevation A</t>
+          <t>LI0000TIMR Irrigation Timer (EA)</t>
         </is>
       </c>
       <c r="F192" s="2" t="n">
-        <v>735</v>
+        <v>121.88</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C193" s="3" t="n">
-        <v>46296</v>
+        <v>46308</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>1816</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>LI0000ZONE Irrigation Per Zone (EA)</t>
         </is>
       </c>
       <c r="F193" s="2" t="n">
-        <v>9330</v>
+        <v>541.13</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C194" s="3" t="n">
-        <v>46296</v>
+        <v>46308</v>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>1816</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>CP0206 - Patio Cover A - Elevation A</t>
+          <t>LLG000BLDR Ground Cover Boulder (EA)</t>
         </is>
       </c>
       <c r="F194" s="2" t="n">
-        <v>526</v>
+        <v>69</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C195" s="3" t="n">
-        <v>46296</v>
+        <v>46308</v>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>1635</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>BED0030 - Bedroom 3/Bath</t>
+          <t>LLG000CR24 Ground Cover 2-4in Cobble Rock (CY)</t>
         </is>
       </c>
       <c r="F195" s="2" t="n">
-        <v>430</v>
+        <v>87.75</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Skyeview - Mesa - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C196" s="3" t="n">
-        <v>46296</v>
+        <v>46308</v>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>1816</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>BED0040 - Bedroom 4/Bath</t>
+          <t>LLG3QIROCK Ground Cover 3/4in Rock (CY)</t>
         </is>
       </c>
       <c r="F196" s="2" t="n">
-        <v>300</v>
+        <v>78.98</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Ishani Ridge (Century Complete)</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C197" s="3" t="n">
-        <v>46153</v>
+        <v>46308</v>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>ALL</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>LLS01GSHRB Shrubs &amp; Plants 1-gallon (EA)</t>
         </is>
       </c>
       <c r="F197" s="2" t="n">
-        <v>2765</v>
-      </c>
-      <c r="G197" t="inlineStr">
-        <is>
-          <t>Price reduced from contract approved by Tony</t>
-        </is>
+        <v>13.5</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C198" s="3" t="n">
-        <v>46023</v>
+        <v>46308</v>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>1663</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>LLS03GSHRB Shrubs &amp; Plants 3-gallon (EA)</t>
         </is>
       </c>
       <c r="F198" s="2" t="n">
-        <v>11550</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C199" s="3" t="n">
-        <v>46023</v>
+        <v>46308</v>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>1663</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>BED0035 - Bedroom 3/Bath Elevation B</t>
+          <t>LLS05GSHRB Shrubs &amp; Plants 5-gallon (EA)</t>
         </is>
       </c>
       <c r="F199" s="2" t="n">
-        <v>439</v>
+        <v>27.79</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C200" s="3" t="n">
-        <v>46023</v>
+        <v>46308</v>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>1663</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>BED0036 - Bedroom 3/Bath Elevation C</t>
+          <t>LLS15GSHRB Shrubs &amp; Plants 15-gallon (EA)</t>
         </is>
       </c>
       <c r="F200" s="2" t="n">
-        <v>439</v>
+        <v>105</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C201" s="3" t="n">
-        <v>46023</v>
+        <v>46308</v>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>1663</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>CP0206 - Patio Cover A - Elevation A</t>
+          <t>LLT01ITREE Tree 1in Caliper (EA)</t>
         </is>
       </c>
       <c r="F201" s="2" t="n">
-        <v>437</v>
+        <v>234</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C202" s="3" t="n">
-        <v>46023</v>
+        <v>46308</v>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>1663</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>CP0207 - Patio Cover A - Elevation B</t>
+          <t>LLT02ITREE Tree 2in Caliper (EA)</t>
         </is>
       </c>
       <c r="F202" s="2" t="n">
-        <v>428</v>
+        <v>850</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Terra</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Unit Pricing</t>
         </is>
       </c>
       <c r="C203" s="3" t="n">
-        <v>46023</v>
+        <v>46308</v>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>1663</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>CP0208 - Patio Cover A - Elevation C</t>
+          <t>LLT03ITREE Tree 3in Caliper (EA)</t>
         </is>
       </c>
       <c r="F203" s="2" t="n">
-        <v>663</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C204" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>1742</t>
+          <t>1635</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="F204" s="2" t="n">
-        <v>11684</v>
+        <v>3534</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C205" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D205" t="inlineStr">
         <is>
@@ -6177,605 +6172,605 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>CP0206 - Patio Cover A - Elevation A</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="F205" s="2" t="n">
-        <v>374</v>
+        <v>3534</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C206" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>1742</t>
+          <t>1816</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>CP0207 - Patio Cover A - Elevation B</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="F206" s="2" t="n">
-        <v>1277</v>
+        <v>3534</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C207" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>1742</t>
+          <t>1635</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>CP0208 - Patio Cover A - Elevation C</t>
+          <t>Pavers</t>
         </is>
       </c>
       <c r="F207" s="2" t="n">
-        <v>1277</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C208" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1635</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>PVO-CP0206 Patio Cover</t>
         </is>
       </c>
       <c r="F208" s="2" t="n">
-        <v>12346</v>
+        <v>725</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C209" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1635</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>CP0206 - Patio Cover A - Elevation A</t>
+          <t>PVO-AL0200 Alumawood Patio Cover - Lattice</t>
         </is>
       </c>
       <c r="F209" s="2" t="n">
-        <v>692</v>
+        <v>725</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C210" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1635</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>CP0207 - Patio Cover A - Elevation B</t>
+          <t>PVO-AL0250 Alumawood Patio Cover - Solid</t>
         </is>
       </c>
       <c r="F210" s="2" t="n">
-        <v>714</v>
+        <v>725</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C211" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1635</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>CP0208 - Patio Cover A - Elevation C</t>
+          <t>PVO-CP155 Patio Pavers Only</t>
         </is>
       </c>
       <c r="F211" s="2" t="n">
-        <v>714</v>
+        <v>725</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>The Bluffs I - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C212" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1742</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>BED0040 - Bedroom 4/Bath</t>
+          <t>Pavers</t>
         </is>
       </c>
       <c r="F212" s="2" t="n">
-        <v>570</v>
+        <v>2703</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C213" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>1863</t>
+          <t>1742</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>PVO-CP0206 Patio Cover</t>
         </is>
       </c>
       <c r="F213" s="2" t="n">
-        <v>12646</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C214" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>1863</t>
+          <t>1742</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>CP0206 - Patio Cover A - Elevation A</t>
+          <t>PVO-AL0200 Alumawood Patio Cover - Lattice</t>
         </is>
       </c>
       <c r="F214" s="2" t="n">
-        <v>720</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C215" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>1863</t>
+          <t>1742</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>CP0207 - Patio Cover A - Elevation B</t>
+          <t>PVO-AL0250 Alumawood Patio Cover - Solid</t>
         </is>
       </c>
       <c r="F215" s="2" t="n">
-        <v>720</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C216" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>1863</t>
+          <t>1742</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>CP0208 - Patio Cover A - Elevation C</t>
+          <t>PVO-CP155 Patio Pavers Only</t>
         </is>
       </c>
       <c r="F216" s="2" t="n">
-        <v>720</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C217" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>1863</t>
+          <t>1816</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>CAS0007 - Guest Quarters w/Direct Access - A</t>
+          <t>Pavers</t>
         </is>
       </c>
       <c r="F217" s="2" t="n">
-        <v>4368</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C218" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>1863</t>
+          <t>1816</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>CAS0008 - Guest Quarters w/Direct Access - B</t>
+          <t>PVO-CP0206 Patio Cover</t>
         </is>
       </c>
       <c r="F218" s="2" t="n">
-        <v>4368</v>
+        <v>825</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C219" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>1863</t>
+          <t>1816</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>CAS0009 - Guest Quarters w/Direct Access - C</t>
+          <t>PVO-AL0200 Alumawood Patio Cover - Lattice</t>
         </is>
       </c>
       <c r="F219" s="2" t="n">
-        <v>4368</v>
+        <v>825</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C220" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>2230</t>
+          <t>1816</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>PVO-AL0250 Alumawood Patio Cover - Solid</t>
         </is>
       </c>
       <c r="F220" s="2" t="n">
-        <v>14023</v>
+        <v>825</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Skyeview - Mesa</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C221" s="3" t="n">
-        <v>46023</v>
+        <v>45748</v>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>2230</t>
+          <t>1816</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>CP0206 - Patio Cover A - Elevation A</t>
+          <t>PVO-CP155 Patio Pavers Only</t>
         </is>
       </c>
       <c r="F221" s="2" t="n">
-        <v>559</v>
+        <v>825</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Union Village</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C222" s="3" t="n">
-        <v>46023</v>
+        <v>45427</v>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>2230</t>
+          <t>1405</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>CP0207 - Patio Cover A - Elevation B</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="F222" s="2" t="n">
-        <v>619</v>
+        <v>547</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Union Village</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C223" s="3" t="n">
-        <v>46023</v>
+        <v>45427</v>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>2230</t>
+          <t>1478</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>CP0208 - Patio Cover A - Elevation C</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="F223" s="2" t="n">
-        <v>657</v>
+        <v>547</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Union Village</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C224" s="3" t="n">
-        <v>46023</v>
+        <v>45427</v>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>2301</t>
+          <t>1478E</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="F224" s="2" t="n">
-        <v>14913</v>
+        <v>547</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Union Village</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C225" s="3" t="n">
-        <v>46023</v>
+        <v>45427</v>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>2301</t>
+          <t>1479</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>CP0206 - Patio Cover A - Elevation A</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="F225" s="2" t="n">
-        <v>720</v>
+        <v>547</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Ishani Ridge (Century Complete)</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C226" s="3" t="n">
-        <v>46023</v>
+        <v>45792</v>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>2301</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>CP0207 - Patio Cover A - Elevation B</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="F226" s="2" t="n">
-        <v>720</v>
+        <v>3210</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>The Bluffs II - Concrete</t>
+          <t>Skyeview - Mesa - Concrete</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6784,26 +6779,26 @@
         </is>
       </c>
       <c r="C227" s="3" t="n">
-        <v>46023</v>
+        <v>46296</v>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>2301</t>
+          <t>1635</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>CP0208 - Patio Cover A - Elevation C</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F227" s="2" t="n">
-        <v>720</v>
+        <v>8567</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Skyeview - Arroyo - Concrete</t>
+          <t>Skyeview - Mesa - Concrete</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6812,26 +6807,26 @@
         </is>
       </c>
       <c r="C228" s="3" t="n">
-        <v>45839</v>
+        <v>46296</v>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Beverly</t>
+          <t>1635</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
         </is>
       </c>
       <c r="F228" s="2" t="n">
-        <v>5273</v>
+        <v>501</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Skyeview - Arroyo - Concrete</t>
+          <t>Skyeview - Mesa - Concrete</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -6840,11 +6835,11 @@
         </is>
       </c>
       <c r="C229" s="3" t="n">
-        <v>45839</v>
+        <v>46296</v>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Captiva</t>
+          <t>1742</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
@@ -6853,13 +6848,13 @@
         </is>
       </c>
       <c r="F229" s="2" t="n">
-        <v>5659</v>
+        <v>8926</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Skyeview - Arroyo - Concrete</t>
+          <t>Skyeview - Mesa - Concrete</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -6868,26 +6863,26 @@
         </is>
       </c>
       <c r="C230" s="3" t="n">
-        <v>45839</v>
+        <v>46296</v>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Delray</t>
+          <t>1742</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
         </is>
       </c>
       <c r="F230" s="2" t="n">
-        <v>5955</v>
+        <v>735</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Skyeview - Arroyo - Concrete</t>
+          <t>Skyeview - Mesa - Concrete</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6896,11 +6891,11 @@
         </is>
       </c>
       <c r="C231" s="3" t="n">
-        <v>45992</v>
+        <v>46296</v>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Beverly</t>
+          <t>1816</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
@@ -6909,13 +6904,13 @@
         </is>
       </c>
       <c r="F231" s="2" t="n">
-        <v>4925</v>
+        <v>9330</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Skyeview - Arroyo - Concrete</t>
+          <t>Skyeview - Mesa - Concrete</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6924,26 +6919,26 @@
         </is>
       </c>
       <c r="C232" s="3" t="n">
-        <v>45992</v>
+        <v>46296</v>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Captiva</t>
+          <t>1816</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
         </is>
       </c>
       <c r="F232" s="2" t="n">
-        <v>5286</v>
+        <v>526</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Skyeview - Arroyo - Concrete</t>
+          <t>Skyeview - Mesa - Concrete</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6952,26 +6947,26 @@
         </is>
       </c>
       <c r="C233" s="3" t="n">
-        <v>45992</v>
+        <v>46296</v>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Delray</t>
+          <t>1635</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>BED0030 - Bedroom 3/Bath</t>
         </is>
       </c>
       <c r="F233" s="2" t="n">
-        <v>5562</v>
+        <v>430</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Skyeview - Arroyo - Concrete</t>
+          <t>Skyeview - Mesa - Concrete</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -6984,50 +6979,55 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>Beverly</t>
+          <t>1816</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>BED0040 - Bedroom 4/Bath</t>
         </is>
       </c>
       <c r="F234" s="2" t="n">
-        <v>4802</v>
+        <v>300</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Skyeview - Arroyo - Concrete</t>
+          <t>Ishani Ridge (Century Complete)</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Plan Pricing</t>
         </is>
       </c>
       <c r="C235" s="3" t="n">
-        <v>46296</v>
+        <v>46153</v>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>Captiva</t>
+          <t>ALL</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="F235" s="2" t="n">
-        <v>5154</v>
+        <v>2765</v>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Price reduced from contract approved by Tony</t>
+        </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Skyeview - Arroyo - Concrete</t>
+          <t>The Bluffs I - Concrete</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -7036,11 +7036,11 @@
         </is>
       </c>
       <c r="C236" s="3" t="n">
-        <v>46296</v>
+        <v>46023</v>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Delray</t>
+          <t>1663</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -7049,103 +7049,1167 @@
         </is>
       </c>
       <c r="F236" s="2" t="n">
-        <v>5423</v>
+        <v>11550</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Edgeview Estates</t>
+          <t>The Bluffs I - Concrete</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="C237" s="3" t="n">
-        <v>46327</v>
+        <v>46023</v>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Vista</t>
+          <t>1663</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>BED0035 - Bedroom 3/Bath Elevation B</t>
         </is>
       </c>
       <c r="F237" s="2" t="n">
-        <v>3306</v>
-      </c>
-      <c r="G237" t="inlineStr">
-        <is>
-          <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
-        </is>
+        <v>439</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Edgeview Estates</t>
+          <t>The Bluffs I - Concrete</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Plan Pricing</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="C238" s="3" t="n">
-        <v>46327</v>
+        <v>46023</v>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Horizon</t>
+          <t>1663</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>BED0036 - Bedroom 3/Bath Elevation C</t>
         </is>
       </c>
       <c r="F238" s="2" t="n">
-        <v>3577</v>
-      </c>
-      <c r="G238" t="inlineStr">
-        <is>
-          <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
-        </is>
+        <v>439</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>1663</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F239" s="2" t="n">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C240" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>1663</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>CP0207 - Patio Cover A - Elevation B</t>
+        </is>
+      </c>
+      <c r="F240" s="2" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C241" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>1663</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>CP0208 - Patio Cover A - Elevation C</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="n">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C242" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>1742</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="n">
+        <v>11684</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C243" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>1742</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="n">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C244" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>1742</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>CP0207 - Patio Cover A - Elevation B</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="n">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C245" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>1742</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>CP0208 - Patio Cover A - Elevation C</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="n">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C246" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>1831</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="n">
+        <v>12346</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C247" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>1831</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="n">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C248" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>1831</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>CP0207 - Patio Cover A - Elevation B</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="n">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C249" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>1831</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>CP0208 - Patio Cover A - Elevation C</t>
+        </is>
+      </c>
+      <c r="F249" s="2" t="n">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>The Bluffs I - Concrete</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C250" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>1831</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>BED0040 - Bedroom 4/Bath</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="n">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C251" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F251" s="2" t="n">
+        <v>12646</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C252" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>CP0207 - Patio Cover A - Elevation B</t>
+        </is>
+      </c>
+      <c r="F253" s="2" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C254" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>CP0208 - Patio Cover A - Elevation C</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C255" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>CAS0007 - Guest Quarters w/Direct Access - A</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="n">
+        <v>4368</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C256" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>CAS0008 - Guest Quarters w/Direct Access - B</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="n">
+        <v>4368</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C257" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>1863</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>CAS0009 - Guest Quarters w/Direct Access - C</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="n">
+        <v>4368</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C258" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>2230</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="n">
+        <v>14023</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>2230</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F259" s="2" t="n">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C260" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>2230</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>CP0207 - Patio Cover A - Elevation B</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="n">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>2230</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>CP0208 - Patio Cover A - Elevation C</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="n">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C262" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="n">
+        <v>14913</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C263" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>CP0206 - Patio Cover A - Elevation A</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C264" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>CP0207 - Patio Cover A - Elevation B</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>The Bluffs II - Concrete</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C265" s="3" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>2301</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>CP0208 - Patio Cover A - Elevation C</t>
+        </is>
+      </c>
+      <c r="F265" s="2" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C266" s="3" t="n">
+        <v>45839</v>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Beverly</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="n">
+        <v>5273</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="n">
+        <v>45839</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Captiva</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F267" s="2" t="n">
+        <v>5659</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C268" s="3" t="n">
+        <v>45839</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Delray</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F268" s="2" t="n">
+        <v>5955</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C269" s="3" t="n">
+        <v>45992</v>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Beverly</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F269" s="2" t="n">
+        <v>4925</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C270" s="3" t="n">
+        <v>45992</v>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Captiva</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="n">
+        <v>5286</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C271" s="3" t="n">
+        <v>45992</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Delray</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F271" s="2" t="n">
+        <v>5562</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C272" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Beverly</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F272" s="2" t="n">
+        <v>4802</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C273" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Captiva</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F273" s="2" t="n">
+        <v>5154</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Skyeview - Arroyo - Concrete</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="C274" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Delray</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="F274" s="2" t="n">
+        <v>5423</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
           <t>Edgeview Estates</t>
         </is>
       </c>
-      <c r="B239" t="inlineStr">
+      <c r="B275" t="inlineStr">
         <is>
           <t>Plan Pricing</t>
         </is>
       </c>
-      <c r="C239" s="3" t="n">
+      <c r="C275" s="3" t="n">
         <v>46327</v>
       </c>
-      <c r="D239" t="inlineStr">
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Vista</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F275" s="2" t="n">
+        <v>3306</v>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Edgeview Estates</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Plan Pricing</t>
+        </is>
+      </c>
+      <c r="C276" s="3" t="n">
+        <v>46327</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Horizon</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="n">
+        <v>3577</v>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Edgeview Estates</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Plan Pricing</t>
+        </is>
+      </c>
+      <c r="C277" s="3" t="n">
+        <v>46327</v>
+      </c>
+      <c r="D277" t="inlineStr">
         <is>
           <t>Summit</t>
         </is>
       </c>
-      <c r="E239" t="inlineStr">
+      <c r="E277" t="inlineStr">
         <is>
           <t>Pavers</t>
         </is>
       </c>
-      <c r="F239" s="2" t="n">
+      <c r="F277" s="2" t="n">
         <v>3140</v>
       </c>
-      <c r="G239" t="inlineStr">
+      <c r="G277" t="inlineStr">
         <is>
           <t>PPS 5002087 Subcontract 00314260, signed 10/21/26</t>
         </is>

</xml_diff>